<commit_message>
updated UI with working insights wordcloud
</commit_message>
<xml_diff>
--- a/static/output/analysis_results.xlsx
+++ b/static/output/analysis_results.xlsx
@@ -491,29 +491,29 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>37.5%</t>
+          <t>75.0%</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H2" t="n">
         <v>16</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>{\"product_id\": \"B0DSKMKJV5\", \"product_name\": \"Samsung Galaxy S25 Ultra 5G AI Smartphone (Titanium Black, 12GB RAM, 512GB Storage), 200MP Camera, S Pen Included, Long Battery Life\", \"product_url\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"summary\": {\"total_reviews\": 16, \"average_rating\": 4.38, \"sentiment_breakdown\": {\"negative\": 6, \"positive\": 6, \"neutral\": 4}, \"overall_sentiment\": \"negative\", \"accuracy_score\": 37.5}, \"reviews\": [{\"author\": \"Nihir Shah\", \"rating\": \"5.0\", \"date\": \"29 Apr 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    The Samsung Galaxy S25 Ultra continues the Ultra legacy with a device that’s powerful, polished, and packed with cutting-edge features. It’s clear Samsung aimed to solidify its position at the top of the premium smartphone market—and it mostly succeeds.Design and DisplayThe S25 Ultra features a 6.9-inch Dynamic AMOLED 2X display with a 120Hz adaptive refresh rate, offering vibrant colors, deep blacks, and smooth scrolling.The display has a resolution of 3120 x 1440 pixels.It is protected by Corning Gorilla Glass Armor 2, which provides enhanced durability.The phone has a titanium frame and an IP68 rating for dust and water resistance.It also includes an embedded S Pen stylus.Software &amp; FeaturesRunning One UI 7.1 based on Android 15, the user experience is smooth and customizable. Samsung’s commitment to 7 years of software updates gives it an edge over most Android competitors. The integration of Galaxy AI, such as real-time translation, generative photo editing, and productivity enhancements in Samsung Notes, brings genuinely useful features to the everyday experience.CameraThe S25 Ultra has a quad-camera setup:200MP wide-angle primary camera50MP ultra-wide-angle camera10MP telephoto camera (3x optical zoom)50MP periscope telephoto camera (5x optical zoom)The front-facing camera is 12MP.The camera system supports 8K video recording, HDR, and various professional features.Performance and HardwareThe S25 Ultra is powered by the Snapdragon 8 Elite processor.It comes with 12GB or 16GB of RAM.Storage options include 256GB, 512GB, and 1TB.The phone runs on Android 15 with Samsung\'s One UI 7.BatteryThe S25 Ultra has a 5000mAh battery.It supports 45W wired fast charging and 15W wireless charging.Other FeaturesThe phone supports 5G connectivity.It has an ultrasonic in-display fingerprint sensor.It includes Wi-Fi 7, Bluetooth 5.3, NFC, and USB Type-C.SummaryThe Samsung Galaxy S25 Ultra is a premium smartphone with a top-of-the-line display, powerful performance, a versatile camera system, and a long-lasting battery. It also has an S Pen, which is useful for productivity and creativity.\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Amazon Customer\", \"rating\": \"5.0\", \"date\": \"07 May 2025\", \"text\": \"I\'ve been using the Galaxy S25 Ultra for over two months now, having upgraded from the S22 Ultra — and I couldn’t be more satisfied. The display is absolutely stunning, offering crisp visuals and vibrant colors that enhance every viewing experience. The camera is top-notch, particularly excelling in low-light photography — easily the best in the industry.Battery life is another strong point; despite my heavy usage, it easily lasts a full day without needing a recharge. Performance-wise, the phone runs incredibly smooth with no lags or slowdowns. Overall, the S25 Ultra is a powerful, well-rounded upgrade that delivers on all front.\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Avishek DeyAvishek Dey\", \"rating\": \"5.0\", \"date\": \"05 Feb 2025\", \"text\": \"I switched to the Galaxy S25 Ultra after using the iPhone 12 Pro Max for 4 years. The display is absolutely stunning, super bright and the colours pop out. S25 Ultra is very snappy, apps open instantly and higher refresh rate makes the animations very smooth. Camera is decent too. Overall a very worthy upgrade from my current phone\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Deepansh J.\", \"rating\": \"4.0\", \"date\": \"03 May 2025\", \"text\": \"Phone is nice.Performance and speed is good.Little heavy in weight.But battery can be improved to 6000 mah.\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"neutral\"}, {\"author\": \"PRADEEP N.\", \"rating\": \"1.0\", \"date\": \"04 Apr 2025\", \"text\": \"Be very careful before ordering expensive phones at seemingly attractive discounts - you might be in for a shock. They might send you a used/second hand set. Which is what happened in my case. I received it on March 27th but it had already been activated on 11th February. Was lucky to find out because I happened to get the warranty checked from a authorised Samsung store. However, to their credit, Amazon agreed to take it back immediately and issue a refund. Now in the process....Disappointed\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Kushagra M.\", \"rating\": \"5.0\", \"date\": \"22 Feb 2025\", \"text\": \"The design, look and feel of the UI, battery, display, multi-tasking and AI functionality is top-notch. Camera, gaming experience, S-pen support is pretty good too. One of the best flagship phone, if not the best one.\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Aman\", \"rating\": \"5.0\", \"date\": \"14 Apr 2025\", \"text\": \"Superb\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"neutral\"}, {\"author\": \"Arun Ganesh\", \"rating\": \"5.0\", \"date\": \"26 Mar 2025\", \"text\": \"I was initially hesitant to purchase the S25 Ultra, but after 2 weeks of use, I\'m thrilled to share my overwhelmingly positive experience!The battery life has been a standout feature for me, consistently lasting a full day and often stretching into the next with moderate to heavy use.The phone\'s overall performance has been seamless, with lightning-fast app loading, effortless multitasking, and silky-smooth graphics.The display is stunning, with vibrant colors and crisp details that make every visual experience a joy.I\'ve also been impressed with the camera\'s capabilities, delivering crisp, high-quality photos and videos in a variety of conditions.Overall, the S25 Ultra has exceeded my expectations and truly lives up to its reputation as an Android powerhouse. If you\'re in the market for a new flagship device, I highly recommend giving this one a serious look!\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Nihir Shah\", \"rating\": \"5.0\", \"date\": \"29 Apr 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    The Samsung Galaxy S25 Ultra continues the Ultra legacy with a device that’s powerful, polished, and packed with cutting-edge features. It’s clear Samsung aimed to solidify its position at the top of the premium smartphone market—and it mostly succeeds.Design and DisplayThe S25 Ultra features a 6.9-inch Dynamic AMOLED 2X display with a 120Hz adaptive refresh rate, offering vibrant colors, deep blacks, and smooth scrolling.The display has a resolution of 3120 x 1440 pixels.It is protected by Corning Gorilla Glass Armor 2, which provides enhanced durability.The phone has a titanium frame and an IP68 rating for dust and water resistance.It also includes an embedded S Pen stylus.Software &amp; FeaturesRunning One UI 7.1 based on Android 15, the user experience is smooth and customizable. Samsung’s commitment to 7 years of software updates gives it an edge over most Android competitors. The integration of Galaxy AI, such as real-time translation, generative photo editing, and productivity enhancements in Samsung Notes, brings genuinely useful features to the everyday experience.CameraThe S25 Ultra has a quad-camera setup:200MP wide-angle primary camera50MP ultra-wide-angle camera10MP telephoto camera (3x optical zoom)50MP periscope telephoto camera (5x optical zoom)The front-facing camera is 12MP.The camera system supports 8K video recording, HDR, and various professional features.Performance and HardwareThe S25 Ultra is powered by the Snapdragon 8 Elite processor.It comes with 12GB or 16GB of RAM.Storage options include 256GB, 512GB, and 1TB.The phone runs on Android 15 with Samsung\'s One UI 7.BatteryThe S25 Ultra has a 5000mAh battery.It supports 45W wired fast charging and 15W wireless charging.Other FeaturesThe phone supports 5G connectivity.It has an ultrasonic in-display fingerprint sensor.It includes Wi-Fi 7, Bluetooth 5.3, NFC, and USB Type-C.SummaryThe Samsung Galaxy S25 Ultra is a premium smartphone with a top-of-the-line display, powerful performance, a versatile camera system, and a long-lasting battery. It also has an S Pen, which is useful for productivity and creativity.\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Amazon Customer\", \"rating\": \"5.0\", \"date\": \"07 May 2025\", \"text\": \"I\'ve been using the Galaxy S25 Ultra for over two months now, having upgraded from the S22 Ultra — and I couldn’t be more satisfied. The display is absolutely stunning, offering crisp visuals and vibrant colors that enhance every viewing experience. The camera is top-notch, particularly excelling in low-light photography — easily the best in the industry.Battery life is another strong point; despite my heavy usage, it easily lasts a full day without needing a recharge. Performance-wise, the phone runs incredibly smooth with no lags or slowdowns. Overall, the S25 Ultra is a powerful, well-rounded upgrade that delivers on all front.\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Avishek DeyAvishek Dey\", \"rating\": \"5.0\", \"date\": \"05 Feb 2025\", \"text\": \"I switched to the Galaxy S25 Ultra after using the iPhone 12 Pro Max for 4 years. The display is absolutely stunning, super bright and the colours pop out. S25 Ultra is very snappy, apps open instantly and higher refresh rate makes the animations very smooth. Camera is decent too. Overall a very worthy upgrade from my current phone\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Deepansh J.\", \"rating\": \"4.0\", \"date\": \"03 May 2025\", \"text\": \"Phone is nice.Performance and speed is good.Little heavy in weight.But battery can be improved to 6000 mah.\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"neutral\"}, {\"author\": \"PRADEEP N.\", \"rating\": \"1.0\", \"date\": \"04 Apr 2025\", \"text\": \"Be very careful before ordering expensive phones at seemingly attractive discounts - you might be in for a shock. They might send you a used/second hand set. Which is what happened in my case. I received it on March 27th but it had already been activated on 11th February. Was lucky to find out because I happened to get the warranty checked from a authorised Samsung store. However, to their credit, Amazon agreed to take it back immediately and issue a refund. Now in the process....Disappointed\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Kushagra M.\", \"rating\": \"5.0\", \"date\": \"22 Feb 2025\", \"text\": \"The design, look and feel of the UI, battery, display, multi-tasking and AI functionality is top-notch. Camera, gaming experience, S-pen support is pretty good too. One of the best flagship phone, if not the best one.\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Aman\", \"rating\": \"5.0\", \"date\": \"14 Apr 2025\", \"text\": \"Superb\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"neutral\"}, {\"author\": \"Arun Ganesh\", \"rating\": \"5.0\", \"date\": \"26 Mar 2025\", \"text\": \"I was initially hesitant to purchase the S25 Ultra, but after 2 weeks of use, I\'m thrilled to share my overwhelmingly positive experience!The battery life has been a standout feature for me, consistently lasting a full day and often stretching into the next with moderate to heavy use.The phone\'s overall performance has been seamless, with lightning-fast app loading, effortless multitasking, and silky-smooth graphics.The display is stunning, with vibrant colors and crisp details that make every visual experience a joy.I\'ve also been impressed with the camera\'s capabilities, delivering crisp, high-quality photos and videos in a variety of conditions.Overall, the S25 Ultra has exceeded my expectations and truly lives up to its reputation as an Android powerhouse. If you\'re in the market for a new flagship device, I highly recommend giving this one a serious look!\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"positive\"}]}</t>
+          <t>{\"product_id\": \"B0DSKMKJV5\", \"product_name\": \"Samsung Galaxy S25 Ultra 5G AI Smartphone (Titanium Black, 12GB RAM, 512GB Storage), 200MP Camera, S Pen Included, Long Battery Life\", \"product_url\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"summary\": {\"total_reviews\": 16, \"average_rating\": 4.38, \"sentiment_breakdown\": {\"positive\": 12, \"neutral\": 2, \"negative\": 2}, \"overall_sentiment\": \"positive\", \"accuracy_score\": 75.0}, \"reviews\": [{\"author\": \"Nihir Shah\", \"rating\": \"5.0\", \"date\": \"29 Apr 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    The Samsung Galaxy S25 Ultra continues the Ultra legacy with a device that’s powerful, polished, and packed with cutting-edge features. It’s clear Samsung aimed to solidify its position at the top of the premium smartphone market—and it mostly succeeds.Design and DisplayThe S25 Ultra features a 6.9-inch Dynamic AMOLED 2X display with a 120Hz adaptive refresh rate, offering vibrant colors, deep blacks, and smooth scrolling.The display has a resolution of 3120 x 1440 pixels.It is protected by Corning Gorilla Glass Armor 2, which provides enhanced durability.The phone has a titanium frame and an IP68 rating for dust and water resistance.It also includes an embedded S Pen stylus.Software &amp; FeaturesRunning One UI 7.1 based on Android 15, the user experience is smooth and customizable. Samsung’s commitment to 7 years of software updates gives it an edge over most Android competitors. The integration of Galaxy AI, such as real-time translation, generative photo editing, and productivity enhancements in Samsung Notes, brings genuinely useful features to the everyday experience.CameraThe S25 Ultra has a quad-camera setup:200MP wide-angle primary camera50MP ultra-wide-angle camera10MP telephoto camera (3x optical zoom)50MP periscope telephoto camera (5x optical zoom)The front-facing camera is 12MP.The camera system supports 8K video recording, HDR, and various professional features.Performance and HardwareThe S25 Ultra is powered by the Snapdragon 8 Elite processor.It comes with 12GB or 16GB of RAM.Storage options include 256GB, 512GB, and 1TB.The phone runs on Android 15 with Samsung\'s One UI 7.BatteryThe S25 Ultra has a 5000mAh battery.It supports 45W wired fast charging and 15W wireless charging.Other FeaturesThe phone supports 5G connectivity.It has an ultrasonic in-display fingerprint sensor.It includes Wi-Fi 7, Bluetooth 5.3, NFC, and USB Type-C.SummaryThe Samsung Galaxy S25 Ultra is a premium smartphone with a top-of-the-line display, powerful performance, a versatile camera system, and a long-lasting battery. It also has an S Pen, which is useful for productivity and creativity.\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Amazon Customer\", \"rating\": \"5.0\", \"date\": \"07 May 2025\", \"text\": \"I\'ve been using the Galaxy S25 Ultra for over two months now, having upgraded from the S22 Ultra — and I couldn’t be more satisfied. The display is absolutely stunning, offering crisp visuals and vibrant colors that enhance every viewing experience. The camera is top-notch, particularly excelling in low-light photography — easily the best in the industry.Battery life is another strong point; despite my heavy usage, it easily lasts a full day without needing a recharge. Performance-wise, the phone runs incredibly smooth with no lags or slowdowns. Overall, the S25 Ultra is a powerful, well-rounded upgrade that delivers on all front.\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Avishek DeyAvishek Dey\", \"rating\": \"5.0\", \"date\": \"05 Feb 2025\", \"text\": \"I switched to the Galaxy S25 Ultra after using the iPhone 12 Pro Max for 4 years. The display is absolutely stunning, super bright and the colours pop out. S25 Ultra is very snappy, apps open instantly and higher refresh rate makes the animations very smooth. Camera is decent too. Overall a very worthy upgrade from my current phone\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Deepansh J.\", \"rating\": \"4.0\", \"date\": \"03 May 2025\", \"text\": \"Phone is nice.Performance and speed is good.Little heavy in weight.But battery can be improved to 6000 mah.\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"neutral\"}, {\"author\": \"PRADEEP N.\", \"rating\": \"1.0\", \"date\": \"04 Apr 2025\", \"text\": \"Be very careful before ordering expensive phones at seemingly attractive discounts - you might be in for a shock. They might send you a used/second hand set. Which is what happened in my case. I received it on March 27th but it had already been activated on 11th February. Was lucky to find out because I happened to get the warranty checked from a authorised Samsung store. However, to their credit, Amazon agreed to take it back immediately and issue a refund. Now in the process....Disappointed\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Kushagra M.\", \"rating\": \"5.0\", \"date\": \"22 Feb 2025\", \"text\": \"The design, look and feel of the UI, battery, display, multi-tasking and AI functionality is top-notch. Camera, gaming experience, S-pen support is pretty good too. One of the best flagship phone, if not the best one.\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Aman\", \"rating\": \"5.0\", \"date\": \"14 Apr 2025\", \"text\": \"Superb\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Arun Ganesh\", \"rating\": \"5.0\", \"date\": \"26 Mar 2025\", \"text\": \"I was initially hesitant to purchase the S25 Ultra, but after 2 weeks of use, I\'m thrilled to share my overwhelmingly positive experience!The battery life has been a standout feature for me, consistently lasting a full day and often stretching into the next with moderate to heavy use.The phone\'s overall performance has been seamless, with lightning-fast app loading, effortless multitasking, and silky-smooth graphics.The display is stunning, with vibrant colors and crisp details that make every visual experience a joy.I\'ve also been impressed with the camera\'s capabilities, delivering crisp, high-quality photos and videos in a variety of conditions.Overall, the S25 Ultra has exceeded my expectations and truly lives up to its reputation as an Android powerhouse. If you\'re in the market for a new flagship device, I highly recommend giving this one a serious look!\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Nihir Shah\", \"rating\": \"5.0\", \"date\": \"29 Apr 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    The Samsung Galaxy S25 Ultra continues the Ultra legacy with a device that’s powerful, polished, and packed with cutting-edge features. It’s clear Samsung aimed to solidify its position at the top of the premium smartphone market—and it mostly succeeds.Design and DisplayThe S25 Ultra features a 6.9-inch Dynamic AMOLED 2X display with a 120Hz adaptive refresh rate, offering vibrant colors, deep blacks, and smooth scrolling.The display has a resolution of 3120 x 1440 pixels.It is protected by Corning Gorilla Glass Armor 2, which provides enhanced durability.The phone has a titanium frame and an IP68 rating for dust and water resistance.It also includes an embedded S Pen stylus.Software &amp; FeaturesRunning One UI 7.1 based on Android 15, the user experience is smooth and customizable. Samsung’s commitment to 7 years of software updates gives it an edge over most Android competitors. The integration of Galaxy AI, such as real-time translation, generative photo editing, and productivity enhancements in Samsung Notes, brings genuinely useful features to the everyday experience.CameraThe S25 Ultra has a quad-camera setup:200MP wide-angle primary camera50MP ultra-wide-angle camera10MP telephoto camera (3x optical zoom)50MP periscope telephoto camera (5x optical zoom)The front-facing camera is 12MP.The camera system supports 8K video recording, HDR, and various professional features.Performance and HardwareThe S25 Ultra is powered by the Snapdragon 8 Elite processor.It comes with 12GB or 16GB of RAM.Storage options include 256GB, 512GB, and 1TB.The phone runs on Android 15 with Samsung\'s One UI 7.BatteryThe S25 Ultra has a 5000mAh battery.It supports 45W wired fast charging and 15W wireless charging.Other FeaturesThe phone supports 5G connectivity.It has an ultrasonic in-display fingerprint sensor.It includes Wi-Fi 7, Bluetooth 5.3, NFC, and USB Type-C.SummaryThe Samsung Galaxy S25 Ultra is a premium smartphone with a top-of-the-line display, powerful performance, a versatile camera system, and a long-lasting battery. It also has an S Pen, which is useful for productivity and creativity.\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Amazon Customer\", \"rating\": \"5.0\", \"date\": \"07 May 2025\", \"text\": \"I\'ve been using the Galaxy S25 Ultra for over two months now, having upgraded from the S22 Ultra — and I couldn’t be more satisfied. The display is absolutely stunning, offering crisp visuals and vibrant colors that enhance every viewing experience. The camera is top-notch, particularly excelling in low-light photography — easily the best in the industry.Battery life is another strong point; despite my heavy usage, it easily lasts a full day without needing a recharge. Performance-wise, the phone runs incredibly smooth with no lags or slowdowns. Overall, the S25 Ultra is a powerful, well-rounded upgrade that delivers on all front.\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Avishek DeyAvishek Dey\", \"rating\": \"5.0\", \"date\": \"05 Feb 2025\", \"text\": \"I switched to the Galaxy S25 Ultra after using the iPhone 12 Pro Max for 4 years. The display is absolutely stunning, super bright and the colours pop out. S25 Ultra is very snappy, apps open instantly and higher refresh rate makes the animations very smooth. Camera is decent too. Overall a very worthy upgrade from my current phone\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Deepansh J.\", \"rating\": \"4.0\", \"date\": \"03 May 2025\", \"text\": \"Phone is nice.Performance and speed is good.Little heavy in weight.But battery can be improved to 6000 mah.\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"neutral\"}, {\"author\": \"PRADEEP N.\", \"rating\": \"1.0\", \"date\": \"04 Apr 2025\", \"text\": \"Be very careful before ordering expensive phones at seemingly attractive discounts - you might be in for a shock. They might send you a used/second hand set. Which is what happened in my case. I received it on March 27th but it had already been activated on 11th February. Was lucky to find out because I happened to get the warranty checked from a authorised Samsung store. However, to their credit, Amazon agreed to take it back immediately and issue a refund. Now in the process....Disappointed\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Kushagra M.\", \"rating\": \"5.0\", \"date\": \"22 Feb 2025\", \"text\": \"The design, look and feel of the UI, battery, display, multi-tasking and AI functionality is top-notch. Camera, gaming experience, S-pen support is pretty good too. One of the best flagship phone, if not the best one.\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Aman\", \"rating\": \"5.0\", \"date\": \"14 Apr 2025\", \"text\": \"Superb\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Arun Ganesh\", \"rating\": \"5.0\", \"date\": \"26 Mar 2025\", \"text\": \"I was initially hesitant to purchase the S25 Ultra, but after 2 weeks of use, I\'m thrilled to share my overwhelmingly positive experience!The battery life has been a standout feature for me, consistently lasting a full day and often stretching into the next with moderate to heavy use.The phone\'s overall performance has been seamless, with lightning-fast app loading, effortless multitasking, and silky-smooth graphics.The display is stunning, with vibrant colors and crisp details that make every visual experience a joy.I\'ve also been impressed with the camera\'s capabilities, delivering crisp, high-quality photos and videos in a variety of conditions.Overall, the S25 Ultra has exceeded my expectations and truly lives up to its reputation as an Android powerhouse. If you\'re in the market for a new flagship device, I highly recommend giving this one a serious look!\n  \nRead more\", \"product_id\": \"B0DSKMKJV5\", \"link\": \"https://www.amazon.in/Samsung-Smartphone-Titanium-Storage-Included/dp/B0DSKMKJV5/ref=sr_1_3?crid=1LYSSGDKQ9KGQ&amp;dib=eyJ2IjoiMSJ9.6F9zxmqbhCO38LI-LW5u6uX5p_i9BhrpRmOubwMF6wjPDIO6VZkyfmdBNJz4oEp1n-wsQhHaCVuyrZXbVnKaX4XlxHTtW-aVZ9kFV_8e8489N8p048SHSJ19GWFAWIIldOyJ0kFxNaZeFqctwXdSfXP94sJV8txJrNV3EqzCtVZ5aIMSBoGMkkcCfY7qtQSOQxyVVP4Qw4B4jcwbD4mqfo9J4Aeck72a52mXj7sjzNk.v2XhDgp1crT3P9vuf34bKRiz-zb-AbcLZ7xiomulUBg&amp;dib_tag=se&amp;keywords=Samsung+Galaxy+S25+Ultra&amp;qid=1748551919&amp;sprefix=samsung+galaxy+s25+ultra,aps,513&amp;sr=8-3\", \"sentiment\": \"positive\"}]}</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -538,24 +538,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
         <v>10</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>{\"product_id\": \"B07WDJMX16\", \"product_name\": \"Vivo X200 Pro 5G (Titanium Grey, 16GB RAM, 512GB Storage) with No Cost EMI/Additional Exchange Offers\", \"product_url\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"summary\": {\"total_reviews\": 10, \"average_rating\": 4.8, \"sentiment_breakdown\": {\"negative\": 4, \"positive\": 6}, \"overall_sentiment\": \"positive\", \"accuracy_score\": 60.0}, \"reviews\": [{\"author\": \"Bappa royBappa roy\", \"rating\": \"5.0\", \"date\": \"17 Jan 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    Pros:- 1. telephoto lense : captures stunning portrait2. Macro shots: The best in the industry of smartphones within the range3. Battery backup: With heavy usage lasts 1day with min 25% charge remaining for useWith standard usage lasts for 1.5 days with ease.4. Fingerprint &amp; face unlock: The smoothest among all used devices till now and best thing is face unlock even works in low light and dark consitions alao.5. Processor: the best in terms of performance in gaming &amp; other tasks.6. RAM management: The best as keeps in the same page while  opened after 3 days in \\"eFootball 2024\\" and many ithers apps.Cons:-1. Bulky: Seems to the bulkiest phone compared to previusly used ones.2. Difficult to hold: The phone is difficult to hold due to huge camera bump and it always feels that is will fall from hand anytime. One hand use has limited excess to whole screen.\n  \nRead more\", \"product_id\": \"B07WDJMX16\", \"link\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"AbhilashAbhilash\", \"rating\": \"5.0\", \"date\": \"04 Feb 2025\", \"text\": \"Camera: Best in the market, significantly better than my previous Samsung S21 Ultra. The 10x, 5x, and 3x zoom are excellent.AI Features: Not on the level of Samsung S24/S25 Ultra.Design: Looks good, but the camera bump doesn’t feel very practical. Still getting used to it after a month.Display: Great quality, no complaints.Sound: Good and clear.UI: A major drawback. Samsung’s One UI is far better in terms of experience.Gaming: Performs well with smooth gameplay.Battery: Good battery life, lasts well through the day.Build &amp; Feel: Slim, compact, and feels premium in hand.IR Blaster: Placed in the camera module instead of on top, but having it is still better than not.Processor: Was initially nervous about the Dimensity chip, but it turned out to be really capable.Social Media Camera Integration: Needs improvement. Vivo should work on better integration like Apple does with Instagram and Snapchat.Overall: Not a perfect phone, but a well-balanced one with the best camera in the market. Haven’t faced any issues so far.\n  \nRead more\", \"product_id\": \"B07WDJMX16\", \"link\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Riyas M\", \"rating\": \"4.0\", \"date\": \"22 May 2025\", \"text\": \"This is phone is really good. I upgraded from an s22 ultra.UI is really not that bad as everyone say. It could be better but it\'s really good on the basics like animation, customisation etc but not on par with oneui 7.The display is also good. Plenty bright and dims very well. Personally not a fan of the color saturation but no complaints here.The sound is good. Rich and loud but the volume levels are not linear.Camera is great ofcourse. Both main and the telephoto. Stunning photos and videos. Vivo has nailed the balance between true to life and rich vibrant colours.Ultra wide is average. Selfie camera is trash.The battery life is not on par with the capacity. This could be improved through updates and the charging speed is acceptable.The Bulld quality isn\'t as great but nothing bad. It doesn\'t feel like a tank when you hold it.Performance is really great. Everything runs without a hassle. Mediatek is better than snappy in terms of sustained performance but this doesn\'t give peak like 8 elite.Vibration motor is okish. Button are also okish. Fingerprint scanner is best in class.Overall pretty good phone with few little downsides.\n  \nRead more\", \"product_id\": \"B07WDJMX16\", \"link\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Vikas MahajanVikas Mahajan\", \"rating\": \"5.0\", \"date\": \"19 Dec 2024\", \"text\": \"Outstanding Phone with DSLR-Like Camera Quality!I recently upgraded to the Vivo X200 Pro, and I couldn’t be happier with my choice. This phone is a complete powerhouse!Pros:Display: The OLED display is vibrant, with excellent brightness and crisp resolution. It’s a treat for watching videos or scrolling through content.Performance: The processor is incredibly fast, handling multitasking and gaming effortlessly without any lags.Camera: The camera quality is phenomenal! It clicks real DSLR-like photos with stunning detail and natural colors, even in low-light conditions. It’s a game-changer for photography enthusiasts.Battery Life: The battery lasts all day, even with heavy usage, and the fast charging is a lifesaver.Design: The sleek and premium design feels great in the hand. It’s stylish yet sturdy.If you’re looking for a top-tier smartphone experience with outstanding camera performance, the Vivo X200 Pro is worth every penny!\n  \nRead more\", \"product_id\": \"B07WDJMX16\", \"link\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"sunilsunil\", \"rating\": \"5.0\", \"date\": \"17 Jan 2025\", \"text\": \"If you want a smartphone for complete camera you won\'t get better one than thisIf you want a smartphone for best battery life you won\'t get better one than thisThe image processing, photo optimization, battery optimisation are far better than what I expectedThe dimensity 9400 Chip is tuned for efficiency more than perfomance you won\'t find any ui lags, u don\'t get any heating issues evening in heavy tasksThis is a battery beast no smartphone in segment can beat the battery life of this phone including S24 ultra and Iphone 16 pro MaxFor 95k this is complete value for money phonePeak Camera 📸, Peak durability, Peak Battery 🔋Worth every pennyConsider buying this if you are a photography geek like me.\n  \nRead more\", \"product_id\": \"B07WDJMX16\", \"link\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Bappa royBappa roy\", \"rating\": \"5.0\", \"date\": \"17 Jan 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    Pros:- 1. telephoto lense : captures stunning portrait2. Macro shots: The best in the industry of smartphones within the range3. Battery backup: With heavy usage lasts 1day with min 25% charge remaining for useWith standard usage lasts for 1.5 days with ease.4. Fingerprint &amp; face unlock: The smoothest among all used devices till now and best thing is face unlock even works in low light and dark consitions alao.5. Processor: the best in terms of performance in gaming &amp; other tasks.6. RAM management: The best as keeps in the same page while  opened after 3 days in \\"eFootball 2024\\" and many ithers apps.Cons:-1. Bulky: Seems to the bulkiest phone compared to previusly used ones.2. Difficult to hold: The phone is difficult to hold due to huge camera bump and it always feels that is will fall from hand anytime. One hand use has limited excess to whole screen.\n  \nRead more\", \"product_id\": \"B07WDJMX16\", \"link\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"AbhilashAbhilash\", \"rating\": \"5.0\", \"date\": \"04 Feb 2025\", \"text\": \"Camera: Best in the market, significantly better than my previous Samsung S21 Ultra. The 10x, 5x, and 3x zoom are excellent.AI Features: Not on the level of Samsung S24/S25 Ultra.Design: Looks good, but the camera bump doesn’t feel very practical. Still getting used to it after a month.Display: Great quality, no complaints.Sound: Good and clear.UI: A major drawback. Samsung’s One UI is far better in terms of experience.Gaming: Performs well with smooth gameplay.Battery: Good battery life, lasts well through the day.Build &amp; Feel: Slim, compact, and feels premium in hand.IR Blaster: Placed in the camera module instead of on top, but having it is still better than not.Processor: Was initially nervous about the Dimensity chip, but it turned out to be really capable.Social Media Camera Integration: Needs improvement. Vivo should work on better integration like Apple does with Instagram and Snapchat.Overall: Not a perfect phone, but a well-balanced one with the best camera in the market. Haven’t faced any issues so far.\n  \nRead more\", \"product_id\": \"B07WDJMX16\", \"link\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Riyas M\", \"rating\": \"4.0\", \"date\": \"22 May 2025\", \"text\": \"This is phone is really good. I upgraded from an s22 ultra.UI is really not that bad as everyone say. It could be better but it\'s really good on the basics like animation, customisation etc but not on par with oneui 7.The display is also good. Plenty bright and dims very well. Personally not a fan of the color saturation but no complaints here.The sound is good. Rich and loud but the volume levels are not linear.Camera is great ofcourse. Both main and the telephoto. Stunning photos and videos. Vivo has nailed the balance between true to life and rich vibrant colours.Ultra wide is average. Selfie camera is trash.The battery life is not on par with the capacity. This could be improved through updates and the charging speed is acceptable.The Bulld quality isn\'t as great but nothing bad. It doesn\'t feel like a tank when you hold it.Performance is really great. Everything runs without a hassle. Mediatek is better than snappy in terms of sustained performance but this doesn\'t give peak like 8 elite.Vibration motor is okish. Button are also okish. Fingerprint scanner is best in class.Overall pretty good phone with few little downsides.\n  \nRead more\", \"product_id\": \"B07WDJMX16\", \"link\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Vikas MahajanVikas Mahajan\", \"rating\": \"5.0\", \"date\": \"19 Dec 2024\", \"text\": \"Outstanding Phone with DSLR-Like Camera Quality!I recently upgraded to the Vivo X200 Pro, and I couldn’t be happier with my choice. This phone is a complete powerhouse!Pros:Display: The OLED display is vibrant, with excellent brightness and crisp resolution. It’s a treat for watching videos or scrolling through content.Performance: The processor is incredibly fast, handling multitasking and gaming effortlessly without any lags.Camera: The camera quality is phenomenal! It clicks real DSLR-like photos with stunning detail and natural colors, even in low-light conditions. It’s a game-changer for photography enthusiasts.Battery Life: The battery lasts all day, even with heavy usage, and the fast charging is a lifesaver.Design: The sleek and premium design feels great in the hand. It’s stylish yet sturdy.If you’re looking for a top-tier smartphone experience with outstanding camera performance, the Vivo X200 Pro is worth every penny!\n  \nRead more\", \"product_id\": \"B07WDJMX16\", \"link\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"sunilsunil\", \"rating\": \"5.0\", \"date\": \"17 Jan 2025\", \"text\": \"If you want a smartphone for complete camera you won\'t get better one than thisIf you want a smartphone for best battery life you won\'t get better one than thisThe image processing, photo optimization, battery optimisation are far better than what I expectedThe dimensity 9400 Chip is tuned for efficiency more than perfomance you won\'t find any ui lags, u don\'t get any heating issues evening in heavy tasksThis is a battery beast no smartphone in segment can beat the battery life of this phone including S24 ultra and Iphone 16 pro MaxFor 95k this is complete value for money phonePeak Camera 📸, Peak durability, Peak Battery 🔋Worth every pennyConsider buying this if you are a photography geek like me.\n  \nRead more\", \"product_id\": \"B07WDJMX16\", \"link\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"sentiment\": \"negative\"}]}</t>
+          <t>{\"product_id\": \"B07WDJMX16\", \"product_name\": \"Vivo X200 Pro 5G (Titanium Grey, 16GB RAM, 512GB Storage) with No Cost EMI/Additional Exchange Offers\", \"product_url\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"summary\": {\"total_reviews\": 10, \"average_rating\": 4.8, \"sentiment_breakdown\": {\"positive\": 10}, \"overall_sentiment\": \"positive\", \"accuracy_score\": 100.0}, \"reviews\": [{\"author\": \"Bappa royBappa roy\", \"rating\": \"5.0\", \"date\": \"17 Jan 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    Pros:- 1. telephoto lense : captures stunning portrait2. Macro shots: The best in the industry of smartphones within the range3. Battery backup: With heavy usage lasts 1day with min 25% charge remaining for useWith standard usage lasts for 1.5 days with ease.4. Fingerprint &amp; face unlock: The smoothest among all used devices till now and best thing is face unlock even works in low light and dark consitions alao.5. Processor: the best in terms of performance in gaming &amp; other tasks.6. RAM management: The best as keeps in the same page while  opened after 3 days in \\"eFootball 2024\\" and many ithers apps.Cons:-1. Bulky: Seems to the bulkiest phone compared to previusly used ones.2. Difficult to hold: The phone is difficult to hold due to huge camera bump and it always feels that is will fall from hand anytime. One hand use has limited excess to whole screen.\n  \nRead more\", \"product_id\": \"B07WDJMX16\", \"link\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"AbhilashAbhilash\", \"rating\": \"5.0\", \"date\": \"04 Feb 2025\", \"text\": \"Camera: Best in the market, significantly better than my previous Samsung S21 Ultra. The 10x, 5x, and 3x zoom are excellent.AI Features: Not on the level of Samsung S24/S25 Ultra.Design: Looks good, but the camera bump doesn’t feel very practical. Still getting used to it after a month.Display: Great quality, no complaints.Sound: Good and clear.UI: A major drawback. Samsung’s One UI is far better in terms of experience.Gaming: Performs well with smooth gameplay.Battery: Good battery life, lasts well through the day.Build &amp; Feel: Slim, compact, and feels premium in hand.IR Blaster: Placed in the camera module instead of on top, but having it is still better than not.Processor: Was initially nervous about the Dimensity chip, but it turned out to be really capable.Social Media Camera Integration: Needs improvement. Vivo should work on better integration like Apple does with Instagram and Snapchat.Overall: Not a perfect phone, but a well-balanced one with the best camera in the market. Haven’t faced any issues so far.\n  \nRead more\", \"product_id\": \"B07WDJMX16\", \"link\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Riyas M\", \"rating\": \"4.0\", \"date\": \"22 May 2025\", \"text\": \"This is phone is really good. I upgraded from an s22 ultra.UI is really not that bad as everyone say. It could be better but it\'s really good on the basics like animation, customisation etc but not on par with oneui 7.The display is also good. Plenty bright and dims very well. Personally not a fan of the color saturation but no complaints here.The sound is good. Rich and loud but the volume levels are not linear.Camera is great ofcourse. Both main and the telephoto. Stunning photos and videos. Vivo has nailed the balance between true to life and rich vibrant colours.Ultra wide is average. Selfie camera is trash.The battery life is not on par with the capacity. This could be improved through updates and the charging speed is acceptable.The Bulld quality isn\'t as great but nothing bad. It doesn\'t feel like a tank when you hold it.Performance is really great. Everything runs without a hassle. Mediatek is better than snappy in terms of sustained performance but this doesn\'t give peak like 8 elite.Vibration motor is okish. Button are also okish. Fingerprint scanner is best in class.Overall pretty good phone with few little downsides.\n  \nRead more\", \"product_id\": \"B07WDJMX16\", \"link\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Vikas MahajanVikas Mahajan\", \"rating\": \"5.0\", \"date\": \"19 Dec 2024\", \"text\": \"Outstanding Phone with DSLR-Like Camera Quality!I recently upgraded to the Vivo X200 Pro, and I couldn’t be happier with my choice. This phone is a complete powerhouse!Pros:Display: The OLED display is vibrant, with excellent brightness and crisp resolution. It’s a treat for watching videos or scrolling through content.Performance: The processor is incredibly fast, handling multitasking and gaming effortlessly without any lags.Camera: The camera quality is phenomenal! It clicks real DSLR-like photos with stunning detail and natural colors, even in low-light conditions. It’s a game-changer for photography enthusiasts.Battery Life: The battery lasts all day, even with heavy usage, and the fast charging is a lifesaver.Design: The sleek and premium design feels great in the hand. It’s stylish yet sturdy.If you’re looking for a top-tier smartphone experience with outstanding camera performance, the Vivo X200 Pro is worth every penny!\n  \nRead more\", \"product_id\": \"B07WDJMX16\", \"link\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"sunilsunil\", \"rating\": \"5.0\", \"date\": \"17 Jan 2025\", \"text\": \"If you want a smartphone for complete camera you won\'t get better one than thisIf you want a smartphone for best battery life you won\'t get better one than thisThe image processing, photo optimization, battery optimisation are far better than what I expectedThe dimensity 9400 Chip is tuned for efficiency more than perfomance you won\'t find any ui lags, u don\'t get any heating issues evening in heavy tasksThis is a battery beast no smartphone in segment can beat the battery life of this phone including S24 ultra and Iphone 16 pro MaxFor 95k this is complete value for money phonePeak Camera 📸, Peak durability, Peak Battery 🔋Worth every pennyConsider buying this if you are a photography geek like me.\n  \nRead more\", \"product_id\": \"B07WDJMX16\", \"link\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Bappa royBappa roy\", \"rating\": \"5.0\", \"date\": \"17 Jan 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    Pros:- 1. telephoto lense : captures stunning portrait2. Macro shots: The best in the industry of smartphones within the range3. Battery backup: With heavy usage lasts 1day with min 25% charge remaining for useWith standard usage lasts for 1.5 days with ease.4. Fingerprint &amp; face unlock: The smoothest among all used devices till now and best thing is face unlock even works in low light and dark consitions alao.5. Processor: the best in terms of performance in gaming &amp; other tasks.6. RAM management: The best as keeps in the same page while  opened after 3 days in \\"eFootball 2024\\" and many ithers apps.Cons:-1. Bulky: Seems to the bulkiest phone compared to previusly used ones.2. Difficult to hold: The phone is difficult to hold due to huge camera bump and it always feels that is will fall from hand anytime. One hand use has limited excess to whole screen.\n  \nRead more\", \"product_id\": \"B07WDJMX16\", \"link\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"AbhilashAbhilash\", \"rating\": \"5.0\", \"date\": \"04 Feb 2025\", \"text\": \"Camera: Best in the market, significantly better than my previous Samsung S21 Ultra. The 10x, 5x, and 3x zoom are excellent.AI Features: Not on the level of Samsung S24/S25 Ultra.Design: Looks good, but the camera bump doesn’t feel very practical. Still getting used to it after a month.Display: Great quality, no complaints.Sound: Good and clear.UI: A major drawback. Samsung’s One UI is far better in terms of experience.Gaming: Performs well with smooth gameplay.Battery: Good battery life, lasts well through the day.Build &amp; Feel: Slim, compact, and feels premium in hand.IR Blaster: Placed in the camera module instead of on top, but having it is still better than not.Processor: Was initially nervous about the Dimensity chip, but it turned out to be really capable.Social Media Camera Integration: Needs improvement. Vivo should work on better integration like Apple does with Instagram and Snapchat.Overall: Not a perfect phone, but a well-balanced one with the best camera in the market. Haven’t faced any issues so far.\n  \nRead more\", \"product_id\": \"B07WDJMX16\", \"link\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Riyas M\", \"rating\": \"4.0\", \"date\": \"22 May 2025\", \"text\": \"This is phone is really good. I upgraded from an s22 ultra.UI is really not that bad as everyone say. It could be better but it\'s really good on the basics like animation, customisation etc but not on par with oneui 7.The display is also good. Plenty bright and dims very well. Personally not a fan of the color saturation but no complaints here.The sound is good. Rich and loud but the volume levels are not linear.Camera is great ofcourse. Both main and the telephoto. Stunning photos and videos. Vivo has nailed the balance between true to life and rich vibrant colours.Ultra wide is average. Selfie camera is trash.The battery life is not on par with the capacity. This could be improved through updates and the charging speed is acceptable.The Bulld quality isn\'t as great but nothing bad. It doesn\'t feel like a tank when you hold it.Performance is really great. Everything runs without a hassle. Mediatek is better than snappy in terms of sustained performance but this doesn\'t give peak like 8 elite.Vibration motor is okish. Button are also okish. Fingerprint scanner is best in class.Overall pretty good phone with few little downsides.\n  \nRead more\", \"product_id\": \"B07WDJMX16\", \"link\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Vikas MahajanVikas Mahajan\", \"rating\": \"5.0\", \"date\": \"19 Dec 2024\", \"text\": \"Outstanding Phone with DSLR-Like Camera Quality!I recently upgraded to the Vivo X200 Pro, and I couldn’t be happier with my choice. This phone is a complete powerhouse!Pros:Display: The OLED display is vibrant, with excellent brightness and crisp resolution. It’s a treat for watching videos or scrolling through content.Performance: The processor is incredibly fast, handling multitasking and gaming effortlessly without any lags.Camera: The camera quality is phenomenal! It clicks real DSLR-like photos with stunning detail and natural colors, even in low-light conditions. It’s a game-changer for photography enthusiasts.Battery Life: The battery lasts all day, even with heavy usage, and the fast charging is a lifesaver.Design: The sleek and premium design feels great in the hand. It’s stylish yet sturdy.If you’re looking for a top-tier smartphone experience with outstanding camera performance, the Vivo X200 Pro is worth every penny!\n  \nRead more\", \"product_id\": \"B07WDJMX16\", \"link\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"sunilsunil\", \"rating\": \"5.0\", \"date\": \"17 Jan 2025\", \"text\": \"If you want a smartphone for complete camera you won\'t get better one than thisIf you want a smartphone for best battery life you won\'t get better one than thisThe image processing, photo optimization, battery optimisation are far better than what I expectedThe dimensity 9400 Chip is tuned for efficiency more than perfomance you won\'t find any ui lags, u don\'t get any heating issues evening in heavy tasksThis is a battery beast no smartphone in segment can beat the battery life of this phone including S24 ultra and Iphone 16 pro MaxFor 95k this is complete value for money phonePeak Camera 📸, Peak durability, Peak Battery 🔋Worth every pennyConsider buying this if you are a photography geek like me.\n  \nRead more\", \"product_id\": \"B07WDJMX16\", \"link\": \"https://www.amazon.in/Titanium-Storage-Additional-Exchange-Offers/dp/B07WDJMX16/ref=sr_1_3?crid=1AMENWB5GO0DY&amp;dib=eyJ2IjoiMSJ9.RW_o5BJcY4Y9WG3FGpJDNY2E7rRbskCmv8HFUmg4n6EViv74acd93v3uxtgVfdbhVM6z7SjbBurkA7pSLQTQfuRw1Ay7dLi6_h0jTqdTYgHGcitGIzlJHHAkTu3a1TOIdZWViQj1lW6yvrg-JBZixt-hLMm9vuDYrLg5fheZ6F4EWzLZD1YnYq4k6STINjwq5959_bqJ_EFSE4T5Ugv2vh86OYG2lhh2qjHrOggU0wQ.v_xGoTBUz1SzSFDlDdfK1T8yuNpLOIlYAz6S-CXzweY&amp;dib_tag=se&amp;keywords=vivo+X200+Pro&amp;qid=1748551943&amp;sprefix=vivo+x200+pro,aps,376&amp;sr=8-3\", \"sentiment\": \"positive\"}]}</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -575,29 +575,29 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>57.14%</t>
+          <t>71.43%</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H4" t="n">
         <v>14</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>{\"product_id\": \"B0DYV4177R\", \"product_name\": \"Xiaomi 15 Ultra (Silver Chrome, 16GB/512GB)| 200 MP Leica-Quad Camera | SD 8 Elite | WQHD+ Quad Curve AMOLED | Hyper AI\", \"product_url\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"summary\": {\"total_reviews\": 14, \"average_rating\": 4.0, \"sentiment_breakdown\": {\"positive\": 6, \"negative\": 8}, \"overall_sentiment\": \"negative\", \"accuracy_score\": 57.14}, \"reviews\": [{\"author\": \"Agniva Pal\", \"rating\": \"5.0\", \"date\": \"09 May 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n\n\n\n\n\n\n\n\n\n\n\n    \n        \n\n        \n        \n            \n        \n\n        \n            \n                \n                        \n                \n                \n                    The media could not be loaded.\n                \n            \n                \n            \n            \n        \n    \n    \n\n\n\n\n\n\n\n\n  \n  \n    Xiaomi has taken strides this time to make sure the camera works. I\'ve been using samsung s22 ultra for 3.5 years before this and the immediate jump was highly visible.The main camera is amazing and works in every condition. I was surprised to see that night videos come out without noise and there are no luminous colorful noise dots on the video. The pictures you shoot are really good and after 3.5 years I\'ve managed to take images of pets without the need to hold them still. The fastshot mode actually works. The 1.5x crop and 2x crop was magical. Since the sensor is big, these crops make it feel like it\'s being shot with an actual 1.5 and 2x lens.The 3x tele, even if reviewers have always said is not good enough, is actually good and shoots really good portrait. Actually all the lenses shoot really good portrait. The videos are also pretty balanced.The 4.3x is a literally a superbbbbb lens and you can literally shoot at 20 to 30x and find usable results. I was surprised at what this \'ai\' tele can do! This is really good if you\'re 20 to 30 metres away from birds/animals. You can use this to shoot nice pics / videos.Please be warned that pictures come out like a mirrorless camera and the color science isn\'t like phones. That is a major reason you\'ll find most reviews to prefer vivo with their polished look. Highlights on skin are supposed to stay if you shoot in direct sun and the sun isn\'t supposed to look round if you shoot it above 45 degrees. I love the fact that computational photography has been dialled down in this phone. You can always do those things in post with any good software. I hate the over processed look and this suffices for my case.Leaving the camera aside, I\'d say this is a really good battery for a flagship. I end the day with around 40 to 50 percent at times, and I\'m a heavy user. I use a lot of camera; like a lot of it. I use a lot of youtube and instagram. I edit photos. I also listen to music at least 3 hours in a day while working. All thing combined I\'m getting a screen on time of more than 8 hours.The phone is absolutely smooth and no complaints there. It\'s been a month and I\'ve not faced even one stutter. I sold off my mi 11 ultra after 2 months of use due to multiple issues. It\'s not the case anymore. I don\'t see any polish difference between samsung and this phone. I can\'t relate to the fact that samsung makes a better experience. People keep talking about it, but I\'m not sure I can relate. But yes, there are things I miss like samsung pay (google pay works on this one though), ultra wide band to search for my smart watch (i just let it ring now), a night mode on the camera (i think xiaomi has been over confident and has not included a night mode. I agree that shots come out really good even without one but including one would be good. And please include an astrophotography mode as well. All it has is auto night mode now. There\'s no dedicated mode).I can\'t find any other deterrents as of now. It\'s good for the price\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Soham S.\", \"rating\": \"5.0\", \"date\": \"15 May 2025\", \"text\": \"Apart from the software experience, this is a phone worth he \\"ultra\\" tag. It gets all the basics right and enhances the experience with several positives:1. The phone build quality is great and it has the heft that brings a premium experience. But this is strictly for big hands.2. The phone performance and smoothness is top of the line with no heating issues and unusual battery drain. Infact battery life has been great with more than 1 day\'s battery with my usage.3. The photography experience with the added accesories is superb and it redefines the phrase \\"The best camera is the one you always have on you\\". Photography with this phone is a joy and a convenience that makes me ditch my Sony camera on short trips.4. No complaints on the connectivity end as well.Overall, this the the most value for money \\"Ultra\\" phone that money can buy in India right now and it leaves behind the iphones and samsungs by a huge leap.\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"js\", \"rating\": \"1.0\", \"date\": \"13 May 2025\", \"text\": \"Don\'t buy this mobile. Something is loose inside the phone after use of 8  days. Now, amazon also don\'t exchange it. Also there is heating issue.\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"nidhin\", \"rating\": \"5.0\", \"date\": \"04 May 2025\", \"text\": \"The Xiaomi 15 Ultra delivers outstanding performance, with one of the best cameras in the flagship segment. It captures detailed, vibrant photos, and its low-light capabilities are impressive. The device handles heavy apps and multitasking smoothly, and the gaming experience is excellent thanks to its powerful chipset and high refresh rate display.However, there\'s a minor lag when switching between camera modes, which could be improved with future updates. Also, the large camera bump on the back makes the phone wobble on flat surfaces—so it\'s definitely a good idea to use a protective case for better grip and stability.Overall, the Xiaomi 15 Ultra is a powerhouse with premium features, ideal for photography enthusiasts and gamers alike.\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"SENTHIL KUMARAN\", \"rating\": \"5.0\", \"date\": \"09 May 2025\", \"text\": \"1) one of the best mobile.2) touch is very smoothly3) camera quality is marvelous.4) battery backup is super 💯\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"MANISH PANCHAL\", \"rating\": \"3.0\", \"date\": \"17 May 2025\", \"text\": \"The Xiaomi 15 Ultra undoubtedly makes a strong statement with its superb camera quality, delivering stunning photos and videos with impressive detail and dynamic range. However, it\'s not without its drawbacks. Videographers might be disappointed by the lower bitrate in Log video, potentially limiting flexibility in post-production. Furthermore, the poor noise cancellation in video recording could be a significant issue for capturing clean audio in noisy environments. The inability to connect the DJI Mic mini via Bluetooth is another frustrating limitation for content creators relying on wireless audio solutions. Finally, reports of battery and heating issues raise concerns about sustained performance and user comfort. While the camera prowess is undeniable, these other aspects need serious consideration.\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"drtechNNo\", \"rating\": \"4.0\", \"date\": \"04 May 2025\", \"text\": \"I came from Vivo X200 Pro just to see if xiaomi did it better in camera this year compared to vivo.  Sadly it falls sorry in everything except UI.UI of vivo(fun touch) is very bland but rest all parameters like camera,  battery,  etc are 10_20 percent better on vivo.Very sad to have spent this much on xiaomi and absolutely no sorry by the company to provide sodas updates to improve anything.The xiaomi hardware may be better but in this age of AI and computational photography it sorely falls behind the race\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Agniva Pal\", \"rating\": \"5.0\", \"date\": \"09 May 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n\n\n\n\n\n\n\n\n\n\n\n    \n        \n\n        \n        \n            \n        \n\n        \n            \n                \n                        \n                \n                \n                    The media could not be loaded.\n                \n            \n                \n            \n            \n        \n    \n    \n\n\n\n\n\n\n\n\n  \n  \n    Xiaomi has taken strides this time to make sure the camera works. I\'ve been using samsung s22 ultra for 3.5 years before this and the immediate jump was highly visible.The main camera is amazing and works in every condition. I was surprised to see that night videos come out without noise and there are no luminous colorful noise dots on the video. The pictures you shoot are really good and after 3.5 years I\'ve managed to take images of pets without the need to hold them still. The fastshot mode actually works. The 1.5x crop and 2x crop was magical. Since the sensor is big, these crops make it feel like it\'s being shot with an actual 1.5 and 2x lens.The 3x tele, even if reviewers have always said is not good enough, is actually good and shoots really good portrait. Actually all the lenses shoot really good portrait. The videos are also pretty balanced.The 4.3x is a literally a superbbbbb lens and you can literally shoot at 20 to 30x and find usable results. I was surprised at what this \'ai\' tele can do! This is really good if you\'re 20 to 30 metres away from birds/animals. You can use this to shoot nice pics / videos.Please be warned that pictures come out like a mirrorless camera and the color science isn\'t like phones. That is a major reason you\'ll find most reviews to prefer vivo with their polished look. Highlights on skin are supposed to stay if you shoot in direct sun and the sun isn\'t supposed to look round if you shoot it above 45 degrees. I love the fact that computational photography has been dialled down in this phone. You can always do those things in post with any good software. I hate the over processed look and this suffices for my case.Leaving the camera aside, I\'d say this is a really good battery for a flagship. I end the day with around 40 to 50 percent at times, and I\'m a heavy user. I use a lot of camera; like a lot of it. I use a lot of youtube and instagram. I edit photos. I also listen to music at least 3 hours in a day while working. All thing combined I\'m getting a screen on time of more than 8 hours.The phone is absolutely smooth and no complaints there. It\'s been a month and I\'ve not faced even one stutter. I sold off my mi 11 ultra after 2 months of use due to multiple issues. It\'s not the case anymore. I don\'t see any polish difference between samsung and this phone. I can\'t relate to the fact that samsung makes a better experience. People keep talking about it, but I\'m not sure I can relate. But yes, there are things I miss like samsung pay (google pay works on this one though), ultra wide band to search for my smart watch (i just let it ring now), a night mode on the camera (i think xiaomi has been over confident and has not included a night mode. I agree that shots come out really good even without one but including one would be good. And please include an astrophotography mode as well. All it has is auto night mode now. There\'s no dedicated mode).I can\'t find any other deterrents as of now. It\'s good for the price\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Soham S.\", \"rating\": \"5.0\", \"date\": \"15 May 2025\", \"text\": \"Apart from the software experience, this is a phone worth he \\"ultra\\" tag. It gets all the basics right and enhances the experience with several positives:1. The phone build quality is great and it has the heft that brings a premium experience. But this is strictly for big hands.2. The phone performance and smoothness is top of the line with no heating issues and unusual battery drain. Infact battery life has been great with more than 1 day\'s battery with my usage.3. The photography experience with the added accesories is superb and it redefines the phrase \\"The best camera is the one you always have on you\\". Photography with this phone is a joy and a convenience that makes me ditch my Sony camera on short trips.4. No complaints on the connectivity end as well.Overall, this the the most value for money \\"Ultra\\" phone that money can buy in India right now and it leaves behind the iphones and samsungs by a huge leap.\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"js\", \"rating\": \"1.0\", \"date\": \"13 May 2025\", \"text\": \"Don\'t buy this mobile. Something is loose inside the phone after use of 8  days. Now, amazon also don\'t exchange it. Also there is heating issue.\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"nidhin\", \"rating\": \"5.0\", \"date\": \"04 May 2025\", \"text\": \"The Xiaomi 15 Ultra delivers outstanding performance, with one of the best cameras in the flagship segment. It captures detailed, vibrant photos, and its low-light capabilities are impressive. The device handles heavy apps and multitasking smoothly, and the gaming experience is excellent thanks to its powerful chipset and high refresh rate display.However, there\'s a minor lag when switching between camera modes, which could be improved with future updates. Also, the large camera bump on the back makes the phone wobble on flat surfaces—so it\'s definitely a good idea to use a protective case for better grip and stability.Overall, the Xiaomi 15 Ultra is a powerhouse with premium features, ideal for photography enthusiasts and gamers alike.\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"SENTHIL KUMARAN\", \"rating\": \"5.0\", \"date\": \"09 May 2025\", \"text\": \"1) one of the best mobile.2) touch is very smoothly3) camera quality is marvelous.4) battery backup is super 💯\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"MANISH PANCHAL\", \"rating\": \"3.0\", \"date\": \"17 May 2025\", \"text\": \"The Xiaomi 15 Ultra undoubtedly makes a strong statement with its superb camera quality, delivering stunning photos and videos with impressive detail and dynamic range. However, it\'s not without its drawbacks. Videographers might be disappointed by the lower bitrate in Log video, potentially limiting flexibility in post-production. Furthermore, the poor noise cancellation in video recording could be a significant issue for capturing clean audio in noisy environments. The inability to connect the DJI Mic mini via Bluetooth is another frustrating limitation for content creators relying on wireless audio solutions. Finally, reports of battery and heating issues raise concerns about sustained performance and user comfort. While the camera prowess is undeniable, these other aspects need serious consideration.\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"drtechNNo\", \"rating\": \"4.0\", \"date\": \"04 May 2025\", \"text\": \"I came from Vivo X200 Pro just to see if xiaomi did it better in camera this year compared to vivo.  Sadly it falls sorry in everything except UI.UI of vivo(fun touch) is very bland but rest all parameters like camera,  battery,  etc are 10_20 percent better on vivo.Very sad to have spent this much on xiaomi and absolutely no sorry by the company to provide sodas updates to improve anything.The xiaomi hardware may be better but in this age of AI and computational photography it sorely falls behind the race\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"negative\"}]}</t>
+          <t>{\"product_id\": \"B0DYV4177R\", \"product_name\": \"Xiaomi 15 Ultra (Silver Chrome, 16GB/512GB)| 200 MP Leica-Quad Camera | SD 8 Elite | WQHD+ Quad Curve AMOLED | Hyper AI\", \"product_url\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"summary\": {\"total_reviews\": 14, \"average_rating\": 4.0, \"sentiment_breakdown\": {\"positive\": 10, \"negative\": 4}, \"overall_sentiment\": \"positive\", \"accuracy_score\": 71.43}, \"reviews\": [{\"author\": \"Agniva Pal\", \"rating\": \"5.0\", \"date\": \"09 May 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n\n\n\n\n\n\n\n\n\n\n\n    \n        \n\n        \n        \n            \n        \n\n        \n            \n                \n                        \n                \n                \n                    The media could not be loaded.\n                \n            \n                \n            \n            \n        \n    \n    \n\n\n\n\n\n\n\n\n  \n  \n    Xiaomi has taken strides this time to make sure the camera works. I\'ve been using samsung s22 ultra for 3.5 years before this and the immediate jump was highly visible.The main camera is amazing and works in every condition. I was surprised to see that night videos come out without noise and there are no luminous colorful noise dots on the video. The pictures you shoot are really good and after 3.5 years I\'ve managed to take images of pets without the need to hold them still. The fastshot mode actually works. The 1.5x crop and 2x crop was magical. Since the sensor is big, these crops make it feel like it\'s being shot with an actual 1.5 and 2x lens.The 3x tele, even if reviewers have always said is not good enough, is actually good and shoots really good portrait. Actually all the lenses shoot really good portrait. The videos are also pretty balanced.The 4.3x is a literally a superbbbbb lens and you can literally shoot at 20 to 30x and find usable results. I was surprised at what this \'ai\' tele can do! This is really good if you\'re 20 to 30 metres away from birds/animals. You can use this to shoot nice pics / videos.Please be warned that pictures come out like a mirrorless camera and the color science isn\'t like phones. That is a major reason you\'ll find most reviews to prefer vivo with their polished look. Highlights on skin are supposed to stay if you shoot in direct sun and the sun isn\'t supposed to look round if you shoot it above 45 degrees. I love the fact that computational photography has been dialled down in this phone. You can always do those things in post with any good software. I hate the over processed look and this suffices for my case.Leaving the camera aside, I\'d say this is a really good battery for a flagship. I end the day with around 40 to 50 percent at times, and I\'m a heavy user. I use a lot of camera; like a lot of it. I use a lot of youtube and instagram. I edit photos. I also listen to music at least 3 hours in a day while working. All thing combined I\'m getting a screen on time of more than 8 hours.The phone is absolutely smooth and no complaints there. It\'s been a month and I\'ve not faced even one stutter. I sold off my mi 11 ultra after 2 months of use due to multiple issues. It\'s not the case anymore. I don\'t see any polish difference between samsung and this phone. I can\'t relate to the fact that samsung makes a better experience. People keep talking about it, but I\'m not sure I can relate. But yes, there are things I miss like samsung pay (google pay works on this one though), ultra wide band to search for my smart watch (i just let it ring now), a night mode on the camera (i think xiaomi has been over confident and has not included a night mode. I agree that shots come out really good even without one but including one would be good. And please include an astrophotography mode as well. All it has is auto night mode now. There\'s no dedicated mode).I can\'t find any other deterrents as of now. It\'s good for the price\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Soham S.\", \"rating\": \"5.0\", \"date\": \"15 May 2025\", \"text\": \"Apart from the software experience, this is a phone worth he \\"ultra\\" tag. It gets all the basics right and enhances the experience with several positives:1. The phone build quality is great and it has the heft that brings a premium experience. But this is strictly for big hands.2. The phone performance and smoothness is top of the line with no heating issues and unusual battery drain. Infact battery life has been great with more than 1 day\'s battery with my usage.3. The photography experience with the added accesories is superb and it redefines the phrase \\"The best camera is the one you always have on you\\". Photography with this phone is a joy and a convenience that makes me ditch my Sony camera on short trips.4. No complaints on the connectivity end as well.Overall, this the the most value for money \\"Ultra\\" phone that money can buy in India right now and it leaves behind the iphones and samsungs by a huge leap.\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"js\", \"rating\": \"1.0\", \"date\": \"13 May 2025\", \"text\": \"Don\'t buy this mobile. Something is loose inside the phone after use of 8  days. Now, amazon also don\'t exchange it. Also there is heating issue.\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"nidhin\", \"rating\": \"5.0\", \"date\": \"04 May 2025\", \"text\": \"The Xiaomi 15 Ultra delivers outstanding performance, with one of the best cameras in the flagship segment. It captures detailed, vibrant photos, and its low-light capabilities are impressive. The device handles heavy apps and multitasking smoothly, and the gaming experience is excellent thanks to its powerful chipset and high refresh rate display.However, there\'s a minor lag when switching between camera modes, which could be improved with future updates. Also, the large camera bump on the back makes the phone wobble on flat surfaces—so it\'s definitely a good idea to use a protective case for better grip and stability.Overall, the Xiaomi 15 Ultra is a powerhouse with premium features, ideal for photography enthusiasts and gamers alike.\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"SENTHIL KUMARAN\", \"rating\": \"5.0\", \"date\": \"09 May 2025\", \"text\": \"1) one of the best mobile.2) touch is very smoothly3) camera quality is marvelous.4) battery backup is super 💯\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"MANISH PANCHAL\", \"rating\": \"3.0\", \"date\": \"17 May 2025\", \"text\": \"The Xiaomi 15 Ultra undoubtedly makes a strong statement with its superb camera quality, delivering stunning photos and videos with impressive detail and dynamic range. However, it\'s not without its drawbacks. Videographers might be disappointed by the lower bitrate in Log video, potentially limiting flexibility in post-production. Furthermore, the poor noise cancellation in video recording could be a significant issue for capturing clean audio in noisy environments. The inability to connect the DJI Mic mini via Bluetooth is another frustrating limitation for content creators relying on wireless audio solutions. Finally, reports of battery and heating issues raise concerns about sustained performance and user comfort. While the camera prowess is undeniable, these other aspects need serious consideration.\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"drtechNNo\", \"rating\": \"4.0\", \"date\": \"04 May 2025\", \"text\": \"I came from Vivo X200 Pro just to see if xiaomi did it better in camera this year compared to vivo.  Sadly it falls sorry in everything except UI.UI of vivo(fun touch) is very bland but rest all parameters like camera,  battery,  etc are 10_20 percent better on vivo.Very sad to have spent this much on xiaomi and absolutely no sorry by the company to provide sodas updates to improve anything.The xiaomi hardware may be better but in this age of AI and computational photography it sorely falls behind the race\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Agniva Pal\", \"rating\": \"5.0\", \"date\": \"09 May 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n\n\n\n\n\n\n\n\n\n\n\n    \n        \n\n        \n        \n            \n        \n\n        \n            \n                \n                        \n                \n                \n                    The media could not be loaded.\n                \n            \n                \n            \n            \n        \n    \n    \n\n\n\n\n\n\n\n\n  \n  \n    Xiaomi has taken strides this time to make sure the camera works. I\'ve been using samsung s22 ultra for 3.5 years before this and the immediate jump was highly visible.The main camera is amazing and works in every condition. I was surprised to see that night videos come out without noise and there are no luminous colorful noise dots on the video. The pictures you shoot are really good and after 3.5 years I\'ve managed to take images of pets without the need to hold them still. The fastshot mode actually works. The 1.5x crop and 2x crop was magical. Since the sensor is big, these crops make it feel like it\'s being shot with an actual 1.5 and 2x lens.The 3x tele, even if reviewers have always said is not good enough, is actually good and shoots really good portrait. Actually all the lenses shoot really good portrait. The videos are also pretty balanced.The 4.3x is a literally a superbbbbb lens and you can literally shoot at 20 to 30x and find usable results. I was surprised at what this \'ai\' tele can do! This is really good if you\'re 20 to 30 metres away from birds/animals. You can use this to shoot nice pics / videos.Please be warned that pictures come out like a mirrorless camera and the color science isn\'t like phones. That is a major reason you\'ll find most reviews to prefer vivo with their polished look. Highlights on skin are supposed to stay if you shoot in direct sun and the sun isn\'t supposed to look round if you shoot it above 45 degrees. I love the fact that computational photography has been dialled down in this phone. You can always do those things in post with any good software. I hate the over processed look and this suffices for my case.Leaving the camera aside, I\'d say this is a really good battery for a flagship. I end the day with around 40 to 50 percent at times, and I\'m a heavy user. I use a lot of camera; like a lot of it. I use a lot of youtube and instagram. I edit photos. I also listen to music at least 3 hours in a day while working. All thing combined I\'m getting a screen on time of more than 8 hours.The phone is absolutely smooth and no complaints there. It\'s been a month and I\'ve not faced even one stutter. I sold off my mi 11 ultra after 2 months of use due to multiple issues. It\'s not the case anymore. I don\'t see any polish difference between samsung and this phone. I can\'t relate to the fact that samsung makes a better experience. People keep talking about it, but I\'m not sure I can relate. But yes, there are things I miss like samsung pay (google pay works on this one though), ultra wide band to search for my smart watch (i just let it ring now), a night mode on the camera (i think xiaomi has been over confident and has not included a night mode. I agree that shots come out really good even without one but including one would be good. And please include an astrophotography mode as well. All it has is auto night mode now. There\'s no dedicated mode).I can\'t find any other deterrents as of now. It\'s good for the price\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Soham S.\", \"rating\": \"5.0\", \"date\": \"15 May 2025\", \"text\": \"Apart from the software experience, this is a phone worth he \\"ultra\\" tag. It gets all the basics right and enhances the experience with several positives:1. The phone build quality is great and it has the heft that brings a premium experience. But this is strictly for big hands.2. The phone performance and smoothness is top of the line with no heating issues and unusual battery drain. Infact battery life has been great with more than 1 day\'s battery with my usage.3. The photography experience with the added accesories is superb and it redefines the phrase \\"The best camera is the one you always have on you\\". Photography with this phone is a joy and a convenience that makes me ditch my Sony camera on short trips.4. No complaints on the connectivity end as well.Overall, this the the most value for money \\"Ultra\\" phone that money can buy in India right now and it leaves behind the iphones and samsungs by a huge leap.\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"js\", \"rating\": \"1.0\", \"date\": \"13 May 2025\", \"text\": \"Don\'t buy this mobile. Something is loose inside the phone after use of 8  days. Now, amazon also don\'t exchange it. Also there is heating issue.\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"nidhin\", \"rating\": \"5.0\", \"date\": \"04 May 2025\", \"text\": \"The Xiaomi 15 Ultra delivers outstanding performance, with one of the best cameras in the flagship segment. It captures detailed, vibrant photos, and its low-light capabilities are impressive. The device handles heavy apps and multitasking smoothly, and the gaming experience is excellent thanks to its powerful chipset and high refresh rate display.However, there\'s a minor lag when switching between camera modes, which could be improved with future updates. Also, the large camera bump on the back makes the phone wobble on flat surfaces—so it\'s definitely a good idea to use a protective case for better grip and stability.Overall, the Xiaomi 15 Ultra is a powerhouse with premium features, ideal for photography enthusiasts and gamers alike.\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"SENTHIL KUMARAN\", \"rating\": \"5.0\", \"date\": \"09 May 2025\", \"text\": \"1) one of the best mobile.2) touch is very smoothly3) camera quality is marvelous.4) battery backup is super 💯\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"MANISH PANCHAL\", \"rating\": \"3.0\", \"date\": \"17 May 2025\", \"text\": \"The Xiaomi 15 Ultra undoubtedly makes a strong statement with its superb camera quality, delivering stunning photos and videos with impressive detail and dynamic range. However, it\'s not without its drawbacks. Videographers might be disappointed by the lower bitrate in Log video, potentially limiting flexibility in post-production. Furthermore, the poor noise cancellation in video recording could be a significant issue for capturing clean audio in noisy environments. The inability to connect the DJI Mic mini via Bluetooth is another frustrating limitation for content creators relying on wireless audio solutions. Finally, reports of battery and heating issues raise concerns about sustained performance and user comfort. While the camera prowess is undeniable, these other aspects need serious consideration.\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"drtechNNo\", \"rating\": \"4.0\", \"date\": \"04 May 2025\", \"text\": \"I came from Vivo X200 Pro just to see if xiaomi did it better in camera this year compared to vivo.  Sadly it falls sorry in everything except UI.UI of vivo(fun touch) is very bland but rest all parameters like camera,  battery,  etc are 10_20 percent better on vivo.Very sad to have spent this much on xiaomi and absolutely no sorry by the company to provide sodas updates to improve anything.The xiaomi hardware may be better but in this age of AI and computational photography it sorely falls behind the race\n  \nRead more\", \"product_id\": \"B0DYV4177R\", \"link\": \"https://www.amazon.in/Xiaomi-Silver-Chrome-Leica-Quad-Camera/dp/B0DYV4177R/ref=sr_1_3?crid=3BFA6EUJA1KBY&amp;dib=eyJ2IjoiMSJ9.SIwGDtLsGB9zcjOAi-WPna8OoNbV1ZjtaKLSccrPQieStqFpMRS9_hILl-YOrjyfMXIRMOcSLY-HVmOdr2KiKExGLDMLhycRMWdd9sP7EiYC4aFvvYSCLHYE7T1rjAAXrGYdHe2VMIYbRGoYQhEOI4BY90flXzumiCik2orxwlEicoe-vqfG0TQ6XjhUqzw57nCbfg1AqO04Vw3AP6dIO0GJ6_F6kd-NREougY5jYbg.eMEs9lMucx0-o1MQhp-JiQCdGqhUOm9iqfjDohdhhq8&amp;dib_tag=se&amp;keywords=Xiaomi+15+Ultra&amp;qid=1748552015&amp;sprefix=xiaomi+15+ultra,aps,359&amp;sr=8-3\", \"sentiment\": \"negative\"}]}</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -617,29 +617,29 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
         <v>12</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>{\"product_id\": \"B0DQ8MJYXF\", \"product_name\": \"OnePlus 13 | Smarter AI | Lifetime Display Warranty (16GB RAM, 512GB Storage Midnight Ocean)\", \"product_url\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"summary\": {\"total_reviews\": 12, \"average_rating\": 4.83, \"sentiment_breakdown\": {\"negative\": 6, \"positive\": 6}, \"overall_sentiment\": \"negative\", \"accuracy_score\": 50.0}, \"reviews\": [{\"author\": \"Dhruthu Meghadooth\", \"rating\": \"5.0\", \"date\": \"26 Apr 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    Everything you could want in a high end phone. It gives you premium build, reliable battery life over a day and half, super fast charging, awesome display and a pretty reliable camera although I did find a bit of over processing in some shots, I do feel like it\'s value for money for what I paid for it which comes around 50k with exchange a steal for that price. Go for it wholeheartedly.\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Nirangkush DasNirangkush Das\", \"rating\": \"5.0\", \"date\": \"30 Mar 2025\", \"text\": \"Disclaimer: My previous android was the realme X2 which I had used since 2019. Hence, I have limited knowledge regarding other android devices/OS. This review is for those people who want to enjoy the experience of a flagship rather than the game-buffs or the photography enthusiasts.Coming to the phone,Performance: Buttery-smooth. Snapdragon 8 Elite is a premium chip. Transitioning between the apps seems so smooth quite like my iphone 13 if not better which I have been using for the last 2 years. I have played Call of Duty in the max settings and the gameplay is very smooth in both Multiplayer and Battle Royal modes. Camera is awesome though I have not used it much.Battery: I have attached battery SS for reference. The silicone battery gives excellent back-up.Build quality: Build quality is very good, quite like a flagship. The screen seems so premium and fluidy.Storage capacity: I have got the 12 GB + 256 GB variant. System &amp; OS takes around 19 GB. One general photo takes around 8-9 MB space.Connectivity: Have found it good particularly the Wifi as compared to my previous phone. It can catch onto weak wifi signal very strongly.OS: Oxygen OS is awesome. The dual tone color looks good.Verdict: Can easily go for it if you need a flagship device on budget when compared to other brand’s flagships (I got it at 65k).\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Joseph kv\", \"rating\": \"5.0\", \"date\": \"19 Mar 2025\", \"text\": \"Title: Flagship Killer! ★★★★★The OnePlus 13 is a powerhouse!✔ Design &amp; Build: Premium feel with a sleek aluminum frame and vegan leather back. IP68/IP69 rated for durability.✔ Display: Stunning 6.82” QHD+ OLED with a 1-120Hz refresh rate—smooth and vibrant.✔ Performance: Snapdragon 8 Elite + advanced cooling = zero lags, even with heavy multitasking.✔ Battery: 6,000mAh lasts 1.5-2 days. 100W fast charging fills up in ~35 minutes!✔ Camera: 50MP triple-camera with Hasselblad tuning—crisp, natural photos.✔ Software: OxygenOS 15 is smooth, with 4 years of updates.Cons: Slightly pricier than previous models; some pre-installed apps can’t be removed.Verdict: A premium flagship with top-tier performance, battery, and cameras. Worth every penny!\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Kedar\", \"rating\": \"4.0\", \"date\": \"05 Feb 2025\", \"text\": \"I had a OnePlus 8 Pro for four and half years. It was a very nice phone having IP 68, wireless charging and Dolby Atmos.The OnePlus 13 stands out as a top-tier Android smartphone, offering a blend of performance, design, and innovation. Its 6.8-inch QHD+ AMOLED display delivers vibrant visuals with a smooth 120Hz refresh rate, ensuring an immersive viewing experience. Powered by Qualcomm\'s Snapdragon 8 Elite processor and up to 16GB of RAM, the device handles multitasking and demanding applications with ease. The triple 50MP rear camera system, developed in collaboration with Hasselblad, captures detailed and color-accurate photos across various lighting conditions. A substantial 6,000mAh battery provides impressive longevity, and with 100W wired fast charging, the phone reaches a full charge swiftly. The inclusion of IP68 and IP69 water resistance, along with MagSafe support, adds to its premium appeal. Running on OxygenOS 15 based on Android 15, the OnePlus 13 offers a clean and responsive user interface. Overall, it presents a compelling package for those seeking a high-end smartphone experience.I am definitely missing Dolby Atmos in this device for sure. Rest everything is fine.\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Shubham S.\", \"rating\": \"5.0\", \"date\": \"21 May 2025\", \"text\": \"Very Great device. Been using this from last 2 months.Performance:Snapdragon 8 elite provides amazing performance.The performance has been top notch, zero lags, hangs and crashes.Camera:The cameras are good, they are almost as good as a flagship.Build:Already stopped phone a few times, it had the factory case, but nothing happened, not even a scratch.Charging:Charging speeds are amazing as well. Both wired and wireless.Display:The display is the out of this world. It is better in all aspects than s25 ultras display except for the anti glare coating.But the display becomes so bright that Idid not even miss the anti glare coating.I have played games during very bright day outdoors on it and I could see the screen like I was indoor.Connectivity:Had zero issues with connectivity. Amazing 5G speeds and coverage compared to my old device.Found few minor bugs in system such as auto brigness does not work sometimes.Camera zoom over modifies the image using AI.\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"PJ.PJ.\", \"rating\": \"5.0\", \"date\": \"14 Apr 2025\", \"text\": \"Given the spec, I found this one overall great phone in android space. Great overall performance so far - fast, smooth, easy cloud sync backup, big battery, robust privacy and security. I had to give a shot to Midnight ocean - the only OP13 which comes with eco leatherette back, as I had bad experience with back glass iphone. Transfer of data was tricky from iphone to android, however using cable it was a breeze in an hour. The only issue I faced in the few days since I got it in my hands was that the animation effects were laggy with first software update but it got fixed with second software update.\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Dhruthu Meghadooth\", \"rating\": \"5.0\", \"date\": \"26 Apr 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    Everything you could want in a high end phone. It gives you premium build, reliable battery life over a day and half, super fast charging, awesome display and a pretty reliable camera although I did find a bit of over processing in some shots, I do feel like it\'s value for money for what I paid for it which comes around 50k with exchange a steal for that price. Go for it wholeheartedly.\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Nirangkush DasNirangkush Das\", \"rating\": \"5.0\", \"date\": \"30 Mar 2025\", \"text\": \"Disclaimer: My previous android was the realme X2 which I had used since 2019. Hence, I have limited knowledge regarding other android devices/OS. This review is for those people who want to enjoy the experience of a flagship rather than the game-buffs or the photography enthusiasts.Coming to the phone,Performance: Buttery-smooth. Snapdragon 8 Elite is a premium chip. Transitioning between the apps seems so smooth quite like my iphone 13 if not better which I have been using for the last 2 years. I have played Call of Duty in the max settings and the gameplay is very smooth in both Multiplayer and Battle Royal modes. Camera is awesome though I have not used it much.Battery: I have attached battery SS for reference. The silicone battery gives excellent back-up.Build quality: Build quality is very good, quite like a flagship. The screen seems so premium and fluidy.Storage capacity: I have got the 12 GB + 256 GB variant. System &amp; OS takes around 19 GB. One general photo takes around 8-9 MB space.Connectivity: Have found it good particularly the Wifi as compared to my previous phone. It can catch onto weak wifi signal very strongly.OS: Oxygen OS is awesome. The dual tone color looks good.Verdict: Can easily go for it if you need a flagship device on budget when compared to other brand’s flagships (I got it at 65k).\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Joseph kv\", \"rating\": \"5.0\", \"date\": \"19 Mar 2025\", \"text\": \"Title: Flagship Killer! ★★★★★The OnePlus 13 is a powerhouse!✔ Design &amp; Build: Premium feel with a sleek aluminum frame and vegan leather back. IP68/IP69 rated for durability.✔ Display: Stunning 6.82” QHD+ OLED with a 1-120Hz refresh rate—smooth and vibrant.✔ Performance: Snapdragon 8 Elite + advanced cooling = zero lags, even with heavy multitasking.✔ Battery: 6,000mAh lasts 1.5-2 days. 100W fast charging fills up in ~35 minutes!✔ Camera: 50MP triple-camera with Hasselblad tuning—crisp, natural photos.✔ Software: OxygenOS 15 is smooth, with 4 years of updates.Cons: Slightly pricier than previous models; some pre-installed apps can’t be removed.Verdict: A premium flagship with top-tier performance, battery, and cameras. Worth every penny!\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Kedar\", \"rating\": \"4.0\", \"date\": \"05 Feb 2025\", \"text\": \"I had a OnePlus 8 Pro for four and half years. It was a very nice phone having IP 68, wireless charging and Dolby Atmos.The OnePlus 13 stands out as a top-tier Android smartphone, offering a blend of performance, design, and innovation. Its 6.8-inch QHD+ AMOLED display delivers vibrant visuals with a smooth 120Hz refresh rate, ensuring an immersive viewing experience. Powered by Qualcomm\'s Snapdragon 8 Elite processor and up to 16GB of RAM, the device handles multitasking and demanding applications with ease. The triple 50MP rear camera system, developed in collaboration with Hasselblad, captures detailed and color-accurate photos across various lighting conditions. A substantial 6,000mAh battery provides impressive longevity, and with 100W wired fast charging, the phone reaches a full charge swiftly. The inclusion of IP68 and IP69 water resistance, along with MagSafe support, adds to its premium appeal. Running on OxygenOS 15 based on Android 15, the OnePlus 13 offers a clean and responsive user interface. Overall, it presents a compelling package for those seeking a high-end smartphone experience.I am definitely missing Dolby Atmos in this device for sure. Rest everything is fine.\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Shubham S.\", \"rating\": \"5.0\", \"date\": \"21 May 2025\", \"text\": \"Very Great device. Been using this from last 2 months.Performance:Snapdragon 8 elite provides amazing performance.The performance has been top notch, zero lags, hangs and crashes.Camera:The cameras are good, they are almost as good as a flagship.Build:Already stopped phone a few times, it had the factory case, but nothing happened, not even a scratch.Charging:Charging speeds are amazing as well. Both wired and wireless.Display:The display is the out of this world. It is better in all aspects than s25 ultras display except for the anti glare coating.But the display becomes so bright that Idid not even miss the anti glare coating.I have played games during very bright day outdoors on it and I could see the screen like I was indoor.Connectivity:Had zero issues with connectivity. Amazing 5G speeds and coverage compared to my old device.Found few minor bugs in system such as auto brigness does not work sometimes.Camera zoom over modifies the image using AI.\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"PJ.PJ.\", \"rating\": \"5.0\", \"date\": \"14 Apr 2025\", \"text\": \"Given the spec, I found this one overall great phone in android space. Great overall performance so far - fast, smooth, easy cloud sync backup, big battery, robust privacy and security. I had to give a shot to Midnight ocean - the only OP13 which comes with eco leatherette back, as I had bad experience with back glass iphone. Transfer of data was tricky from iphone to android, however using cable it was a breeze in an hour. The only issue I faced in the few days since I got it in my hands was that the animation effects were laggy with first software update but it got fixed with second software update.\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"negative\"}]}</t>
+          <t>{\"product_id\": \"B0DQ8MJYXF\", \"product_name\": \"OnePlus 13 | Smarter AI | Lifetime Display Warranty (16GB RAM, 512GB Storage Midnight Ocean)\", \"product_url\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"summary\": {\"total_reviews\": 12, \"average_rating\": 4.83, \"sentiment_breakdown\": {\"positive\": 12}, \"overall_sentiment\": \"positive\", \"accuracy_score\": 100.0}, \"reviews\": [{\"author\": \"Dhruthu Meghadooth\", \"rating\": \"5.0\", \"date\": \"26 Apr 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    Everything you could want in a high end phone. It gives you premium build, reliable battery life over a day and half, super fast charging, awesome display and a pretty reliable camera although I did find a bit of over processing in some shots, I do feel like it\'s value for money for what I paid for it which comes around 50k with exchange a steal for that price. Go for it wholeheartedly.\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Nirangkush DasNirangkush Das\", \"rating\": \"5.0\", \"date\": \"30 Mar 2025\", \"text\": \"Disclaimer: My previous android was the realme X2 which I had used since 2019. Hence, I have limited knowledge regarding other android devices/OS. This review is for those people who want to enjoy the experience of a flagship rather than the game-buffs or the photography enthusiasts.Coming to the phone,Performance: Buttery-smooth. Snapdragon 8 Elite is a premium chip. Transitioning between the apps seems so smooth quite like my iphone 13 if not better which I have been using for the last 2 years. I have played Call of Duty in the max settings and the gameplay is very smooth in both Multiplayer and Battle Royal modes. Camera is awesome though I have not used it much.Battery: I have attached battery SS for reference. The silicone battery gives excellent back-up.Build quality: Build quality is very good, quite like a flagship. The screen seems so premium and fluidy.Storage capacity: I have got the 12 GB + 256 GB variant. System &amp; OS takes around 19 GB. One general photo takes around 8-9 MB space.Connectivity: Have found it good particularly the Wifi as compared to my previous phone. It can catch onto weak wifi signal very strongly.OS: Oxygen OS is awesome. The dual tone color looks good.Verdict: Can easily go for it if you need a flagship device on budget when compared to other brand’s flagships (I got it at 65k).\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Joseph kv\", \"rating\": \"5.0\", \"date\": \"19 Mar 2025\", \"text\": \"Title: Flagship Killer! ★★★★★The OnePlus 13 is a powerhouse!✔ Design &amp; Build: Premium feel with a sleek aluminum frame and vegan leather back. IP68/IP69 rated for durability.✔ Display: Stunning 6.82” QHD+ OLED with a 1-120Hz refresh rate—smooth and vibrant.✔ Performance: Snapdragon 8 Elite + advanced cooling = zero lags, even with heavy multitasking.✔ Battery: 6,000mAh lasts 1.5-2 days. 100W fast charging fills up in ~35 minutes!✔ Camera: 50MP triple-camera with Hasselblad tuning—crisp, natural photos.✔ Software: OxygenOS 15 is smooth, with 4 years of updates.Cons: Slightly pricier than previous models; some pre-installed apps can’t be removed.Verdict: A premium flagship with top-tier performance, battery, and cameras. Worth every penny!\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Kedar\", \"rating\": \"4.0\", \"date\": \"05 Feb 2025\", \"text\": \"I had a OnePlus 8 Pro for four and half years. It was a very nice phone having IP 68, wireless charging and Dolby Atmos.The OnePlus 13 stands out as a top-tier Android smartphone, offering a blend of performance, design, and innovation. Its 6.8-inch QHD+ AMOLED display delivers vibrant visuals with a smooth 120Hz refresh rate, ensuring an immersive viewing experience. Powered by Qualcomm\'s Snapdragon 8 Elite processor and up to 16GB of RAM, the device handles multitasking and demanding applications with ease. The triple 50MP rear camera system, developed in collaboration with Hasselblad, captures detailed and color-accurate photos across various lighting conditions. A substantial 6,000mAh battery provides impressive longevity, and with 100W wired fast charging, the phone reaches a full charge swiftly. The inclusion of IP68 and IP69 water resistance, along with MagSafe support, adds to its premium appeal. Running on OxygenOS 15 based on Android 15, the OnePlus 13 offers a clean and responsive user interface. Overall, it presents a compelling package for those seeking a high-end smartphone experience.I am definitely missing Dolby Atmos in this device for sure. Rest everything is fine.\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Shubham S.\", \"rating\": \"5.0\", \"date\": \"21 May 2025\", \"text\": \"Very Great device. Been using this from last 2 months.Performance:Snapdragon 8 elite provides amazing performance.The performance has been top notch, zero lags, hangs and crashes.Camera:The cameras are good, they are almost as good as a flagship.Build:Already stopped phone a few times, it had the factory case, but nothing happened, not even a scratch.Charging:Charging speeds are amazing as well. Both wired and wireless.Display:The display is the out of this world. It is better in all aspects than s25 ultras display except for the anti glare coating.But the display becomes so bright that Idid not even miss the anti glare coating.I have played games during very bright day outdoors on it and I could see the screen like I was indoor.Connectivity:Had zero issues with connectivity. Amazing 5G speeds and coverage compared to my old device.Found few minor bugs in system such as auto brigness does not work sometimes.Camera zoom over modifies the image using AI.\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"PJ.PJ.\", \"rating\": \"5.0\", \"date\": \"14 Apr 2025\", \"text\": \"Given the spec, I found this one overall great phone in android space. Great overall performance so far - fast, smooth, easy cloud sync backup, big battery, robust privacy and security. I had to give a shot to Midnight ocean - the only OP13 which comes with eco leatherette back, as I had bad experience with back glass iphone. Transfer of data was tricky from iphone to android, however using cable it was a breeze in an hour. The only issue I faced in the few days since I got it in my hands was that the animation effects were laggy with first software update but it got fixed with second software update.\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Dhruthu Meghadooth\", \"rating\": \"5.0\", \"date\": \"26 Apr 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    Everything you could want in a high end phone. It gives you premium build, reliable battery life over a day and half, super fast charging, awesome display and a pretty reliable camera although I did find a bit of over processing in some shots, I do feel like it\'s value for money for what I paid for it which comes around 50k with exchange a steal for that price. Go for it wholeheartedly.\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Nirangkush DasNirangkush Das\", \"rating\": \"5.0\", \"date\": \"30 Mar 2025\", \"text\": \"Disclaimer: My previous android was the realme X2 which I had used since 2019. Hence, I have limited knowledge regarding other android devices/OS. This review is for those people who want to enjoy the experience of a flagship rather than the game-buffs or the photography enthusiasts.Coming to the phone,Performance: Buttery-smooth. Snapdragon 8 Elite is a premium chip. Transitioning between the apps seems so smooth quite like my iphone 13 if not better which I have been using for the last 2 years. I have played Call of Duty in the max settings and the gameplay is very smooth in both Multiplayer and Battle Royal modes. Camera is awesome though I have not used it much.Battery: I have attached battery SS for reference. The silicone battery gives excellent back-up.Build quality: Build quality is very good, quite like a flagship. The screen seems so premium and fluidy.Storage capacity: I have got the 12 GB + 256 GB variant. System &amp; OS takes around 19 GB. One general photo takes around 8-9 MB space.Connectivity: Have found it good particularly the Wifi as compared to my previous phone. It can catch onto weak wifi signal very strongly.OS: Oxygen OS is awesome. The dual tone color looks good.Verdict: Can easily go for it if you need a flagship device on budget when compared to other brand’s flagships (I got it at 65k).\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Joseph kv\", \"rating\": \"5.0\", \"date\": \"19 Mar 2025\", \"text\": \"Title: Flagship Killer! ★★★★★The OnePlus 13 is a powerhouse!✔ Design &amp; Build: Premium feel with a sleek aluminum frame and vegan leather back. IP68/IP69 rated for durability.✔ Display: Stunning 6.82” QHD+ OLED with a 1-120Hz refresh rate—smooth and vibrant.✔ Performance: Snapdragon 8 Elite + advanced cooling = zero lags, even with heavy multitasking.✔ Battery: 6,000mAh lasts 1.5-2 days. 100W fast charging fills up in ~35 minutes!✔ Camera: 50MP triple-camera with Hasselblad tuning—crisp, natural photos.✔ Software: OxygenOS 15 is smooth, with 4 years of updates.Cons: Slightly pricier than previous models; some pre-installed apps can’t be removed.Verdict: A premium flagship with top-tier performance, battery, and cameras. Worth every penny!\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Kedar\", \"rating\": \"4.0\", \"date\": \"05 Feb 2025\", \"text\": \"I had a OnePlus 8 Pro for four and half years. It was a very nice phone having IP 68, wireless charging and Dolby Atmos.The OnePlus 13 stands out as a top-tier Android smartphone, offering a blend of performance, design, and innovation. Its 6.8-inch QHD+ AMOLED display delivers vibrant visuals with a smooth 120Hz refresh rate, ensuring an immersive viewing experience. Powered by Qualcomm\'s Snapdragon 8 Elite processor and up to 16GB of RAM, the device handles multitasking and demanding applications with ease. The triple 50MP rear camera system, developed in collaboration with Hasselblad, captures detailed and color-accurate photos across various lighting conditions. A substantial 6,000mAh battery provides impressive longevity, and with 100W wired fast charging, the phone reaches a full charge swiftly. The inclusion of IP68 and IP69 water resistance, along with MagSafe support, adds to its premium appeal. Running on OxygenOS 15 based on Android 15, the OnePlus 13 offers a clean and responsive user interface. Overall, it presents a compelling package for those seeking a high-end smartphone experience.I am definitely missing Dolby Atmos in this device for sure. Rest everything is fine.\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Shubham S.\", \"rating\": \"5.0\", \"date\": \"21 May 2025\", \"text\": \"Very Great device. Been using this from last 2 months.Performance:Snapdragon 8 elite provides amazing performance.The performance has been top notch, zero lags, hangs and crashes.Camera:The cameras are good, they are almost as good as a flagship.Build:Already stopped phone a few times, it had the factory case, but nothing happened, not even a scratch.Charging:Charging speeds are amazing as well. Both wired and wireless.Display:The display is the out of this world. It is better in all aspects than s25 ultras display except for the anti glare coating.But the display becomes so bright that Idid not even miss the anti glare coating.I have played games during very bright day outdoors on it and I could see the screen like I was indoor.Connectivity:Had zero issues with connectivity. Amazing 5G speeds and coverage compared to my old device.Found few minor bugs in system such as auto brigness does not work sometimes.Camera zoom over modifies the image using AI.\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"PJ.PJ.\", \"rating\": \"5.0\", \"date\": \"14 Apr 2025\", \"text\": \"Given the spec, I found this one overall great phone in android space. Great overall performance so far - fast, smooth, easy cloud sync backup, big battery, robust privacy and security. I had to give a shot to Midnight ocean - the only OP13 which comes with eco leatherette back, as I had bad experience with back glass iphone. Transfer of data was tricky from iphone to android, however using cable it was a breeze in an hour. The only issue I faced in the few days since I got it in my hands was that the animation effects were laggy with first software update but it got fixed with second software update.\n  \nRead more\", \"product_id\": \"B0DQ8MJYXF\", \"link\": \"https://www.amazon.in/OnePlus-13-512GB-Midnight-Ocean/dp/B0DQ8MJYXF/ref=sr_1_3?crid=JVJRW7NMRVIP&amp;dib=eyJ2IjoiMSJ9.ATeYA3KrH9Wb0fbjsbUzvtebcejt3UeUtsz2bSnFdjZYuLZBvPtXKM4JIBLI-ht0IIJ7nHMgy7FCuP-pORHia87pzib1pOvGjv4nb7ZTrqtWuOOJzoukimXDo-l1LC_z6dhpr2BQJEqQz77X7qvpDhekxkm0TO02vMcjqNGLaG23Vzq9-SHIatBT6p63iomGiONoZRyuLO7meIrvwtD2BuKQtDbHVNYz1oy-mCmruqo.uyLDm6GazzMGSo91Vn7lbg0r6sgkbQmiHFaIQl19I84&amp;dib_tag=se&amp;keywords=OnePlus+13&amp;qid=1748552079&amp;sprefix=oneplus+13,aps,457&amp;sr=8-3\", \"sentiment\": \"positive\"}]}</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -655,21 +655,21 @@
         </is>
       </c>
       <c r="B6" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
         <v>4</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>2</v>
-      </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
@@ -677,11 +677,11 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>{\"product_id\": \"B0F5HVFVKH\", \"product_name\": \"Motorola razr 60 Ultra (Pantone Scarab, 16 GB RAM, 512 GB Storage) | Moto AI | Snapdragon® 8 Elite Mobile Platform | 6.9\\" AMOLED 165Hz Display | 50 MP + 50 MP + 50MP Triple Camera\", \"product_url\": \"https://www.amazon.in/Motorola-razr-60-Ultra-Snapdragon%C2%AE/dp/B0F5HVFVKH/ref=sr_1_3?crid=2TMI2QFCK8A8Z&amp;dib=eyJ2IjoiMSJ9.tKCy0Zp_GAMheDynKgHIKQdV9qz4L1fD3DZDQQhhswY8mlPoCpplfNktf4VUGAfGLCxlcOtf_1ZzPnuhWmxKmiRpLE7i6jY1d-DqR0BxBLlvBMfzgRZEirdESJ3UL-mtgttGySVhoXKEppbruoAsAurLddH6JqfCkxounMBnu950XDmY9mShgErmWowuYWbEBe4ylBxByIZceHSy1eFLF4QEEzqJsryemKLK09aXN8E.uk9Yi-AdiOEX1x37cMYYfHi8bLDw3r-OA7cS4Llvon0&amp;dib_tag=se&amp;keywords=Motorola+Razr+60+Ultra&amp;qid=1748552120&amp;sprefix=motorola+razr+60+ultra,aps,529&amp;sr=8-3\", \"summary\": {\"total_reviews\": 2, \"average_rating\": 4.0, \"sentiment_breakdown\": {\"positive\": 2}, \"overall_sentiment\": \"positive\", \"accuracy_score\": 100.0}, \"reviews\": [{\"author\": \"Kamal Kundu\", \"rating\": \"4.0\", \"date\": \"25 May 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    Phone is awesome but eSim option is not active in India. Let me know if there are ways to activate eSim for it.\n  \nRead more\", \"product_id\": \"B0F5HVFVKH\", \"link\": \"https://www.amazon.in/Motorola-razr-60-Ultra-Snapdragon%C2%AE/dp/B0F5HVFVKH/ref=sr_1_3?crid=2TMI2QFCK8A8Z&amp;dib=eyJ2IjoiMSJ9.tKCy0Zp_GAMheDynKgHIKQdV9qz4L1fD3DZDQQhhswY8mlPoCpplfNktf4VUGAfGLCxlcOtf_1ZzPnuhWmxKmiRpLE7i6jY1d-DqR0BxBLlvBMfzgRZEirdESJ3UL-mtgttGySVhoXKEppbruoAsAurLddH6JqfCkxounMBnu950XDmY9mShgErmWowuYWbEBe4ylBxByIZceHSy1eFLF4QEEzqJsryemKLK09aXN8E.uk9Yi-AdiOEX1x37cMYYfHi8bLDw3r-OA7cS4Llvon0&amp;dib_tag=se&amp;keywords=Motorola+Razr+60+Ultra&amp;qid=1748552120&amp;sprefix=motorola+razr+60+ultra,aps,529&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Kamal Kundu\", \"rating\": \"4.0\", \"date\": \"25 May 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    Phone is awesome but eSim option is not active in India. Let me know if there are ways to activate eSim for it.\n  \nRead more\", \"product_id\": \"B0F5HVFVKH\", \"link\": \"https://www.amazon.in/Motorola-razr-60-Ultra-Snapdragon%C2%AE/dp/B0F5HVFVKH/ref=sr_1_3?crid=2TMI2QFCK8A8Z&amp;dib=eyJ2IjoiMSJ9.tKCy0Zp_GAMheDynKgHIKQdV9qz4L1fD3DZDQQhhswY8mlPoCpplfNktf4VUGAfGLCxlcOtf_1ZzPnuhWmxKmiRpLE7i6jY1d-DqR0BxBLlvBMfzgRZEirdESJ3UL-mtgttGySVhoXKEppbruoAsAurLddH6JqfCkxounMBnu950XDmY9mShgErmWowuYWbEBe4ylBxByIZceHSy1eFLF4QEEzqJsryemKLK09aXN8E.uk9Yi-AdiOEX1x37cMYYfHi8bLDw3r-OA7cS4Llvon0&amp;dib_tag=se&amp;keywords=Motorola+Razr+60+Ultra&amp;qid=1748552120&amp;sprefix=motorola+razr+60+ultra,aps,529&amp;sr=8-3\", \"sentiment\": \"positive\"}]}</t>
+          <t>{\"product_id\": \"B0F5HVFVKH\", \"product_name\": \"Motorola razr 60 Ultra (Pantone Scarab, 16 GB RAM, 512 GB Storage) | Moto AI | Snapdragon® 8 Elite Mobile Platform | 6.9\\" AMOLED 165Hz Display | 50 MP + 50 MP + 50MP Triple Camera\", \"product_url\": \"https://www.amazon.in/Motorola-razr-60-Ultra-Snapdragon%C2%AE/dp/B0F5HVFVKH/ref=sr_1_3?crid=2TMI2QFCK8A8Z&amp;dib=eyJ2IjoiMSJ9.tKCy0Zp_GAMheDynKgHIKQdV9qz4L1fD3DZDQQhhswY8mlPoCpplfNktf4VUGAfGLCxlcOtf_1ZzPnuhWmxKmiRpLE7i6jY1d-DqR0BxBLlvBMfzgRZEirdESJ3UL-mtgttGySVhoXKEppbruoAsAurLddH6JqfCkxounMBnu950XDmY9mShgErmWowuYWbEBe4ylBxByIZceHSy1eFLF4QEEzqJsryemKLK09aXN8E.uk9Yi-AdiOEX1x37cMYYfHi8bLDw3r-OA7cS4Llvon0&amp;dib_tag=se&amp;keywords=Motorola+Razr+60+Ultra&amp;qid=1748552120&amp;sprefix=motorola+razr+60+ultra,aps,529&amp;sr=8-3\", \"summary\": {\"total_reviews\": 4, \"average_rating\": 4.5, \"sentiment_breakdown\": {\"positive\": 4}, \"overall_sentiment\": \"positive\", \"accuracy_score\": 100.0}, \"reviews\": [{\"author\": \"Kamal Kundu\", \"rating\": \"4.0\", \"date\": \"25 May 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    Phone is awesome but eSim option is not active in India. Let me know if there are ways to activate eSim for it.\n  \nRead more\", \"product_id\": \"B0F5HVFVKH\", \"link\": \"https://www.amazon.in/Motorola-razr-60-Ultra-Snapdragon%C2%AE/dp/B0F5HVFVKH/ref=sr_1_3?crid=2TMI2QFCK8A8Z&amp;dib=eyJ2IjoiMSJ9.tKCy0Zp_GAMheDynKgHIKQdV9qz4L1fD3DZDQQhhswY8mlPoCpplfNktf4VUGAfGLCxlcOtf_1ZzPnuhWmxKmiRpLE7i6jY1d-DqR0BxBLlvBMfzgRZEirdESJ3UL-mtgttGySVhoXKEppbruoAsAurLddH6JqfCkxounMBnu950XDmY9mShgErmWowuYWbEBe4ylBxByIZceHSy1eFLF4QEEzqJsryemKLK09aXN8E.uk9Yi-AdiOEX1x37cMYYfHi8bLDw3r-OA7cS4Llvon0&amp;dib_tag=se&amp;keywords=Motorola+Razr+60+Ultra&amp;qid=1748552120&amp;sprefix=motorola+razr+60+ultra,aps,529&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Abhijeet Chinchole\", \"rating\": \"5.0\", \"date\": \"28 May 2025\", \"text\": \"This is my very first smartphone, and after using the Moto Razr 60 Ultra for a week, I can confidently say I’m impressed! The design is sleek and premium, and the flip form factor adds a cool, nostalgic touch while still feeling modern.Performance has been smooth so far – apps open quickly, multitasking is easy, and the external display is actually very handy for quick glances or controls without unfolding the phone. The inner screen is vibrant and responsive, making everyday use a joy.Battery life could be better – it gets me through the day, but not much more. That’s the only area where I feel there’s room for improvement.Overall, it’s a fantastic flip phone for anyone who wants something unique yet functional. I’m really enjoying the experience!\n  \nRead more\", \"product_id\": \"B0F5HVFVKH\", \"link\": \"https://www.amazon.in/Motorola-razr-60-Ultra-Snapdragon%C2%AE/dp/B0F5HVFVKH/ref=sr_1_3?crid=2TMI2QFCK8A8Z&amp;dib=eyJ2IjoiMSJ9.tKCy0Zp_GAMheDynKgHIKQdV9qz4L1fD3DZDQQhhswY8mlPoCpplfNktf4VUGAfGLCxlcOtf_1ZzPnuhWmxKmiRpLE7i6jY1d-DqR0BxBLlvBMfzgRZEirdESJ3UL-mtgttGySVhoXKEppbruoAsAurLddH6JqfCkxounMBnu950XDmY9mShgErmWowuYWbEBe4ylBxByIZceHSy1eFLF4QEEzqJsryemKLK09aXN8E.uk9Yi-AdiOEX1x37cMYYfHi8bLDw3r-OA7cS4Llvon0&amp;dib_tag=se&amp;keywords=Motorola+Razr+60+Ultra&amp;qid=1748552120&amp;sprefix=motorola+razr+60+ultra,aps,529&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Kamal Kundu\", \"rating\": \"4.0\", \"date\": \"25 May 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    Phone is awesome but eSim option is not active in India. Let me know if there are ways to activate eSim for it.\n  \nRead more\", \"product_id\": \"B0F5HVFVKH\", \"link\": \"https://www.amazon.in/Motorola-razr-60-Ultra-Snapdragon%C2%AE/dp/B0F5HVFVKH/ref=sr_1_3?crid=2TMI2QFCK8A8Z&amp;dib=eyJ2IjoiMSJ9.tKCy0Zp_GAMheDynKgHIKQdV9qz4L1fD3DZDQQhhswY8mlPoCpplfNktf4VUGAfGLCxlcOtf_1ZzPnuhWmxKmiRpLE7i6jY1d-DqR0BxBLlvBMfzgRZEirdESJ3UL-mtgttGySVhoXKEppbruoAsAurLddH6JqfCkxounMBnu950XDmY9mShgErmWowuYWbEBe4ylBxByIZceHSy1eFLF4QEEzqJsryemKLK09aXN8E.uk9Yi-AdiOEX1x37cMYYfHi8bLDw3r-OA7cS4Llvon0&amp;dib_tag=se&amp;keywords=Motorola+Razr+60+Ultra&amp;qid=1748552120&amp;sprefix=motorola+razr+60+ultra,aps,529&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Abhijeet Chinchole\", \"rating\": \"5.0\", \"date\": \"28 May 2025\", \"text\": \"This is my very first smartphone, and after using the Moto Razr 60 Ultra for a week, I can confidently say I’m impressed! The design is sleek and premium, and the flip form factor adds a cool, nostalgic touch while still feeling modern.Performance has been smooth so far – apps open quickly, multitasking is easy, and the external display is actually very handy for quick glances or controls without unfolding the phone. The inner screen is vibrant and responsive, making everyday use a joy.Battery life could be better – it gets me through the day, but not much more. That’s the only area where I feel there’s room for improvement.Overall, it’s a fantastic flip phone for anyone who wants something unique yet functional. I’m really enjoying the experience!\n  \nRead more\", \"product_id\": \"B0F5HVFVKH\", \"link\": \"https://www.amazon.in/Motorola-razr-60-Ultra-Snapdragon%C2%AE/dp/B0F5HVFVKH/ref=sr_1_3?crid=2TMI2QFCK8A8Z&amp;dib=eyJ2IjoiMSJ9.tKCy0Zp_GAMheDynKgHIKQdV9qz4L1fD3DZDQQhhswY8mlPoCpplfNktf4VUGAfGLCxlcOtf_1ZzPnuhWmxKmiRpLE7i6jY1d-DqR0BxBLlvBMfzgRZEirdESJ3UL-mtgttGySVhoXKEppbruoAsAurLddH6JqfCkxounMBnu950XDmY9mShgErmWowuYWbEBe4ylBxByIZceHSy1eFLF4QEEzqJsryemKLK09aXN8E.uk9Yi-AdiOEX1x37cMYYfHi8bLDw3r-OA7cS4Llvon0&amp;dib_tag=se&amp;keywords=Motorola+Razr+60+Ultra&amp;qid=1748552120&amp;sprefix=motorola+razr+60+ultra,aps,529&amp;sr=8-3\", \"sentiment\": \"positive\"}]}</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -706,24 +706,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>62.5%</t>
+          <t>87.5%</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
         <v>2</v>
-      </c>
-      <c r="G7" t="n">
-        <v>4</v>
       </c>
       <c r="H7" t="n">
         <v>16</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>{\"product_id\": \"B0DZNP1MN3\", \"product_name\": \"Nothing Phone (3A) 5G (White, 8GB RAM, 256GB Storage)\", \"product_url\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"summary\": {\"total_reviews\": 16, \"average_rating\": 4.25, \"sentiment_breakdown\": {\"positive\": 10, \"negative\": 4, \"neutral\": 2}, \"overall_sentiment\": \"positive\", \"accuracy_score\": 62.5}, \"reviews\": [{\"author\": \"Shashwat Shashwat\", \"rating\": \"5.0\", \"date\": \"20 Mar 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    Ordered this for my younger sister, Well i was very curious at first as all the sellers were new &amp; selling at slightly cheaper rates than official, but I checked everything thoroughly, packing was top notch, checked the device on nothing\'s website by IMEI if it was pre activated or what, but fortunately everything was fine. Phone is also nice, decent cameras, Nice UI, but I feel like it get\'s little warm to touch sometimes don\'t know why, Battery is okay too, not very good though but overall seriously it\'s a value for money indeed but yes you need to get a charger seperately as it doesn\'t come with one so keep that in mind, although my sister is very happy.\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Rajan Thakur\", \"rating\": \"4.0\", \"date\": \"13 Apr 2025\", \"text\": \"Overall a great phone with smooth performance and a premium look. Display is crisp, but I found the screen lighting color a bit different compared to Samsung—takes a little time to adjust. Battery and camera are good, and it\'s definitely worth the price. Just a few small things from making it perfect!\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Farhan\", \"rating\": \"5.0\", \"date\": \"17 May 2025\", \"text\": \"Excellent productsExcellent quality of phoneCamera is so clean and awesomeBudget phonePackaging is low but excellent\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Dhiman\", \"rating\": \"1.0\", \"date\": \"27 May 2025\", \"text\": \"Worst decision.Better to buy a brick at this price.Guys trust me the battery wont last u even 4 hours.overnight the battery is going to drain at least 15 percent.Go for motorala edge 60 fusion.Donot repeat my mistake.Tried nothing for the first time.Pathetic brand.\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"negative\"}, {\"author\": \"sunilkumarnella\", \"rating\": \"5.0\", \"date\": \"25 May 2025\", \"text\": \"200%  satisfied\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"neutral\"}, {\"author\": \"Eren Yeager Eren Yeager\", \"rating\": \"5.0\", \"date\": \"09 Apr 2025\", \"text\": \"It\'s slick and beautiful tons of minimal features.... I prefer to use a back cover or tempered glass at back.... And you can trust amazon no damages and battery life is also best\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Deep B.\", \"rating\": \"4.0\", \"date\": \"22 May 2025\", \"text\": \"Good, reasonably fast, cleanly designed phone. The battery isn\'t best in class, but enough for a daily driver.Not for gaming or high intensity usage. Bit large especially with a case, but I prefer that.\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"negative\"}, {\"author\": \"Sudhir waman\", \"rating\": \"5.0\", \"date\": \"16 May 2025\", \"text\": \"Excellent specs\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Shashwat Shashwat\", \"rating\": \"5.0\", \"date\": \"20 Mar 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    Ordered this for my younger sister, Well i was very curious at first as all the sellers were new &amp; selling at slightly cheaper rates than official, but I checked everything thoroughly, packing was top notch, checked the device on nothing\'s website by IMEI if it was pre activated or what, but fortunately everything was fine. Phone is also nice, decent cameras, Nice UI, but I feel like it get\'s little warm to touch sometimes don\'t know why, Battery is okay too, not very good though but overall seriously it\'s a value for money indeed but yes you need to get a charger seperately as it doesn\'t come with one so keep that in mind, although my sister is very happy.\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Rajan Thakur\", \"rating\": \"4.0\", \"date\": \"13 Apr 2025\", \"text\": \"Overall a great phone with smooth performance and a premium look. Display is crisp, but I found the screen lighting color a bit different compared to Samsung—takes a little time to adjust. Battery and camera are good, and it\'s definitely worth the price. Just a few small things from making it perfect!\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Farhan\", \"rating\": \"5.0\", \"date\": \"17 May 2025\", \"text\": \"Excellent productsExcellent quality of phoneCamera is so clean and awesomeBudget phonePackaging is low but excellent\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Dhiman\", \"rating\": \"1.0\", \"date\": \"27 May 2025\", \"text\": \"Worst decision.Better to buy a brick at this price.Guys trust me the battery wont last u even 4 hours.overnight the battery is going to drain at least 15 percent.Go for motorala edge 60 fusion.Donot repeat my mistake.Tried nothing for the first time.Pathetic brand.\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"negative\"}, {\"author\": \"sunilkumarnella\", \"rating\": \"5.0\", \"date\": \"25 May 2025\", \"text\": \"200%  satisfied\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"neutral\"}, {\"author\": \"Eren Yeager Eren Yeager\", \"rating\": \"5.0\", \"date\": \"09 Apr 2025\", \"text\": \"It\'s slick and beautiful tons of minimal features.... I prefer to use a back cover or tempered glass at back.... And you can trust amazon no damages and battery life is also best\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Deep B.\", \"rating\": \"4.0\", \"date\": \"22 May 2025\", \"text\": \"Good, reasonably fast, cleanly designed phone. The battery isn\'t best in class, but enough for a daily driver.Not for gaming or high intensity usage. Bit large especially with a case, but I prefer that.\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"negative\"}, {\"author\": \"Sudhir waman\", \"rating\": \"5.0\", \"date\": \"16 May 2025\", \"text\": \"Excellent specs\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}]}</t>
+          <t>{\"product_id\": \"B0DZNP1MN3\", \"product_name\": \"Nothing Phone (3A) 5G (White, 8GB RAM, 256GB Storage)\", \"product_url\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"summary\": {\"total_reviews\": 16, \"average_rating\": 4.25, \"sentiment_breakdown\": {\"positive\": 14, \"negative\": 2}, \"overall_sentiment\": \"positive\", \"accuracy_score\": 87.5}, \"reviews\": [{\"author\": \"Shashwat Shashwat\", \"rating\": \"5.0\", \"date\": \"20 Mar 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    Ordered this for my younger sister, Well i was very curious at first as all the sellers were new &amp; selling at slightly cheaper rates than official, but I checked everything thoroughly, packing was top notch, checked the device on nothing\'s website by IMEI if it was pre activated or what, but fortunately everything was fine. Phone is also nice, decent cameras, Nice UI, but I feel like it get\'s little warm to touch sometimes don\'t know why, Battery is okay too, not very good though but overall seriously it\'s a value for money indeed but yes you need to get a charger seperately as it doesn\'t come with one so keep that in mind, although my sister is very happy.\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Farhan\", \"rating\": \"5.0\", \"date\": \"17 May 2025\", \"text\": \"Excellent productsExcellent quality of phoneCamera is so clean and awesomeBudget phonePackaging is low but excellent\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Rajan Thakur\", \"rating\": \"4.0\", \"date\": \"13 Apr 2025\", \"text\": \"Overall a great phone with smooth performance and a premium look. Display is crisp, but I found the screen lighting color a bit different compared to Samsung—takes a little time to adjust. Battery and camera are good, and it\'s definitely worth the price. Just a few small things from making it perfect!\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Dhiman\", \"rating\": \"1.0\", \"date\": \"27 May 2025\", \"text\": \"Worst decision.Better to buy a brick at this price.Guys trust me the battery wont last u even 4 hours.overnight the battery is going to drain at least 15 percent.Go for motorala edge 60 fusion.Donot repeat my mistake.Tried nothing for the first time.Pathetic brand.\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"negative\"}, {\"author\": \"sunilkumarnella\", \"rating\": \"5.0\", \"date\": \"25 May 2025\", \"text\": \"200%  satisfied\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Eren Yeager Eren Yeager\", \"rating\": \"5.0\", \"date\": \"09 Apr 2025\", \"text\": \"It\'s slick and beautiful tons of minimal features.... I prefer to use a back cover or tempered glass at back.... And you can trust amazon no damages and battery life is also best\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Sudhir waman\", \"rating\": \"5.0\", \"date\": \"16 May 2025\", \"text\": \"Excellent specs\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Deep B.\", \"rating\": \"4.0\", \"date\": \"22 May 2025\", \"text\": \"Good, reasonably fast, cleanly designed phone. The battery isn\'t best in class, but enough for a daily driver.Not for gaming or high intensity usage. Bit large especially with a case, but I prefer that.\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Shashwat Shashwat\", \"rating\": \"5.0\", \"date\": \"20 Mar 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    Ordered this for my younger sister, Well i was very curious at first as all the sellers were new &amp; selling at slightly cheaper rates than official, but I checked everything thoroughly, packing was top notch, checked the device on nothing\'s website by IMEI if it was pre activated or what, but fortunately everything was fine. Phone is also nice, decent cameras, Nice UI, but I feel like it get\'s little warm to touch sometimes don\'t know why, Battery is okay too, not very good though but overall seriously it\'s a value for money indeed but yes you need to get a charger seperately as it doesn\'t come with one so keep that in mind, although my sister is very happy.\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Farhan\", \"rating\": \"5.0\", \"date\": \"17 May 2025\", \"text\": \"Excellent productsExcellent quality of phoneCamera is so clean and awesomeBudget phonePackaging is low but excellent\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Rajan Thakur\", \"rating\": \"4.0\", \"date\": \"13 Apr 2025\", \"text\": \"Overall a great phone with smooth performance and a premium look. Display is crisp, but I found the screen lighting color a bit different compared to Samsung—takes a little time to adjust. Battery and camera are good, and it\'s definitely worth the price. Just a few small things from making it perfect!\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Dhiman\", \"rating\": \"1.0\", \"date\": \"27 May 2025\", \"text\": \"Worst decision.Better to buy a brick at this price.Guys trust me the battery wont last u even 4 hours.overnight the battery is going to drain at least 15 percent.Go for motorala edge 60 fusion.Donot repeat my mistake.Tried nothing for the first time.Pathetic brand.\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"negative\"}, {\"author\": \"sunilkumarnella\", \"rating\": \"5.0\", \"date\": \"25 May 2025\", \"text\": \"200%  satisfied\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Eren Yeager Eren Yeager\", \"rating\": \"5.0\", \"date\": \"09 Apr 2025\", \"text\": \"It\'s slick and beautiful tons of minimal features.... I prefer to use a back cover or tempered glass at back.... And you can trust amazon no damages and battery life is also best\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Sudhir waman\", \"rating\": \"5.0\", \"date\": \"16 May 2025\", \"text\": \"Excellent specs\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}, {\"author\": \"Deep B.\", \"rating\": \"4.0\", \"date\": \"22 May 2025\", \"text\": \"Good, reasonably fast, cleanly designed phone. The battery isn\'t best in class, but enough for a daily driver.Not for gaming or high intensity usage. Bit large especially with a case, but I prefer that.\n  \nRead more\", \"product_id\": \"B0DZNP1MN3\", \"link\": \"https://www.amazon.in/Nothing-Phone-White-256GB-Storage/dp/B0DZNP1MN3/ref=sr_1_2?crid=28KDOARO7T5AB&amp;dib=eyJ2IjoiMSJ9.k4LDU1LEvT_DhwCVqJxo_OU04GRP-iBZbw7WF59DYJmmsDs_-8sGogafJ3PWggWVwm7u0ZZuG5mjfDgwZKVERNOyOyEIu_31NNHQhQAQ-nwRHok4G_WSuoTOBDRnIN0DIPNlfun7WovlP6FcHcU60F15THPi_Ce4gvUycMIMDwKjmacKheVUB1mfFPd9PCV1BWqncjQoN-Z7UEjTXpHHCRjktsYNxG3sKJWsw0d9Pgc.1-uK6re4x09tFzUk6VoIDs9mPizwua3TcAAMzzAey6Q&amp;dib_tag=se&amp;keywords=nothing+phone+3a&amp;qid=1748537458&amp;sprefix=nothi,aps,246&amp;sr=8-2\", \"sentiment\": \"positive\"}]}</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4.12</v>
+        <v>4.38</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -748,24 +748,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>62.5%</t>
+          <t>87.5%</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H8" t="n">
         <v>16</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>{\"product_id\": \"B0DHL7YT5S\", \"product_name\": \"Samsung Galaxy S24 FE 5G AI Smartphone (Graphite, 8GB RAM, 128GB Storage)\", \"product_url\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"summary\": {\"total_reviews\": 16, \"average_rating\": 4.12, \"sentiment_breakdown\": {\"positive\": 10, \"negative\": 6}, \"overall_sentiment\": \"positive\", \"accuracy_score\": 62.5}, \"reviews\": [{\"author\": \"Gangadhar\", \"rating\": \"5.0\", \"date\": \"06 May 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    Exceptional photo quality great processerBest in the segment display most optimized software  value got money in this price range.Great fast charging no noticeable heating issues but gets temperature\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Thomas\", \"rating\": \"5.0\", \"date\": \"16 May 2025\", \"text\": \"Bought it for 35kTotally worth it for 35k a phone with flagship features camera is very nice you get 4k recording on all 4 camera for this price it\'s pretty rare but on one UI 6.1 it had some heating issue but after updating to oneui7 it stopped heating so much it has far far better heat mangement than s23fe and also chin is slightly thick but most of the time you won\'t notice it gaming is smooth and I get 60fps most of the time you get extrem plus on bgmi\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Abhishek katoch\", \"rating\": \"4.0\", \"date\": \"18 May 2025\", \"text\": \"Device is really good . The only issue is heating\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Annappa\", \"rating\": \"1.0\", \"date\": \"22 May 2025\", \"text\": \"Please don\'t buy these expensive mobiles from Amazon, After paying hell amount of money, you need to run behind service centres for new phone service.\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Ramiz mariner\", \"rating\": \"5.0\", \"date\": \"04 Mar 2025\", \"text\": \"Writing the review after 10 days of usage.Phone Quality - quality is just awesome, looks premium.Size- this matters person to person, honestly I love to have phone size of 5.5 or even 5.0, but know you don\'t get such small size Phone. Coming back to this, I am 5.10 ft, so for my hand this mobile looks big, unable to use with one hand.Performance- have played games continously, watched champions trophy.. Performance is very good...Battery life - it good enough to survive for all day.Weight- again this comes person to person, I l9ve the weight of this cell phone, quiet heavy....\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"RAAZ PATHAN\", \"rating\": \"5.0\", \"date\": \"20 May 2025\", \"text\": \"awesome smoothness to new galaxy ai feautersall package this phoneVALU FOR MONEYI DONT HAVE ANY WORDS\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Vilas N Patil\", \"rating\": \"5.0\", \"date\": \"26 May 2025\", \"text\": \"Nice product and received all items as required\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Abhijit\", \"rating\": \"3.0\", \"date\": \"09 Apr 2025\", \"text\": \"Don\'t fall for this trap. Phone looks good and camera is also pretty decent. Battery also OK for my kind of usage. But it has HEATING ISSUES...No matter whether you close all the apps or what kind of usage you do, it heats up. I don\'t play games, normal browsing also you can feel on your palms despite using a Spigen cover. Without cover it feels even more.DONT GO FOR IT. Buy Iqoo 12 or one plus 13R or Vivo V40 or any other phone...\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Gangadhar\", \"rating\": \"5.0\", \"date\": \"06 May 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    Exceptional photo quality great processerBest in the segment display most optimized software  value got money in this price range.Great fast charging no noticeable heating issues but gets temperature\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Thomas\", \"rating\": \"5.0\", \"date\": \"16 May 2025\", \"text\": \"Bought it for 35kTotally worth it for 35k a phone with flagship features camera is very nice you get 4k recording on all 4 camera for this price it\'s pretty rare but on one UI 6.1 it had some heating issue but after updating to oneui7 it stopped heating so much it has far far better heat mangement than s23fe and also chin is slightly thick but most of the time you won\'t notice it gaming is smooth and I get 60fps most of the time you get extrem plus on bgmi\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Abhishek katoch\", \"rating\": \"4.0\", \"date\": \"18 May 2025\", \"text\": \"Device is really good . The only issue is heating\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Annappa\", \"rating\": \"1.0\", \"date\": \"22 May 2025\", \"text\": \"Please don\'t buy these expensive mobiles from Amazon, After paying hell amount of money, you need to run behind service centres for new phone service.\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Ramiz mariner\", \"rating\": \"5.0\", \"date\": \"04 Mar 2025\", \"text\": \"Writing the review after 10 days of usage.Phone Quality - quality is just awesome, looks premium.Size- this matters person to person, honestly I love to have phone size of 5.5 or even 5.0, but know you don\'t get such small size Phone. Coming back to this, I am 5.10 ft, so for my hand this mobile looks big, unable to use with one hand.Performance- have played games continously, watched champions trophy.. Performance is very good...Battery life - it good enough to survive for all day.Weight- again this comes person to person, I l9ve the weight of this cell phone, quiet heavy....\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"RAAZ PATHAN\", \"rating\": \"5.0\", \"date\": \"20 May 2025\", \"text\": \"awesome smoothness to new galaxy ai feautersall package this phoneVALU FOR MONEYI DONT HAVE ANY WORDS\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Vilas N Patil\", \"rating\": \"5.0\", \"date\": \"26 May 2025\", \"text\": \"Nice product and received all items as required\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Abhijit\", \"rating\": \"3.0\", \"date\": \"09 Apr 2025\", \"text\": \"Don\'t fall for this trap. Phone looks good and camera is also pretty decent. Battery also OK for my kind of usage. But it has HEATING ISSUES...No matter whether you close all the apps or what kind of usage you do, it heats up. I don\'t play games, normal browsing also you can feel on your palms despite using a Spigen cover. Without cover it feels even more.DONT GO FOR IT. Buy Iqoo 12 or one plus 13R or Vivo V40 or any other phone...\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"negative\"}]}</t>
+          <t>{\"product_id\": \"B0DHL7YT5S\", \"product_name\": \"Samsung Galaxy S24 FE 5G AI Smartphone (Graphite, 8GB RAM, 128GB Storage)\", \"product_url\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"summary\": {\"total_reviews\": 16, \"average_rating\": 4.38, \"sentiment_breakdown\": {\"positive\": 14, \"negative\": 2}, \"overall_sentiment\": \"positive\", \"accuracy_score\": 87.5}, \"reviews\": [{\"author\": \"Gangadhar\", \"rating\": \"5.0\", \"date\": \"06 May 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    Exceptional photo quality great processerBest in the segment display most optimized software  value got money in this price range.Great fast charging no noticeable heating issues but gets temperature\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Thomas\", \"rating\": \"5.0\", \"date\": \"16 May 2025\", \"text\": \"Bought it for 35kTotally worth it for 35k a phone with flagship features camera is very nice you get 4k recording on all 4 camera for this price it\'s pretty rare but on one UI 6.1 it had some heating issue but after updating to oneui7 it stopped heating so much it has far far better heat mangement than s23fe and also chin is slightly thick but most of the time you won\'t notice it gaming is smooth and I get 60fps most of the time you get extrem plus on bgmi\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Abhishek katoch\", \"rating\": \"4.0\", \"date\": \"18 May 2025\", \"text\": \"Device is really good . The only issue is heating\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Annappa\", \"rating\": \"1.0\", \"date\": \"22 May 2025\", \"text\": \"Please don\'t buy these expensive mobiles from Amazon, After paying hell amount of money, you need to run behind service centres for new phone service.\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Ramiz mariner\", \"rating\": \"5.0\", \"date\": \"04 Mar 2025\", \"text\": \"Writing the review after 10 days of usage.Phone Quality - quality is just awesome, looks premium.Size- this matters person to person, honestly I love to have phone size of 5.5 or even 5.0, but know you don\'t get such small size Phone. Coming back to this, I am 5.10 ft, so for my hand this mobile looks big, unable to use with one hand.Performance- have played games continously, watched champions trophy.. Performance is very good...Battery life - it good enough to survive for all day.Weight- again this comes person to person, I l9ve the weight of this cell phone, quiet heavy....\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"RAAZ PATHAN\", \"rating\": \"5.0\", \"date\": \"20 May 2025\", \"text\": \"awesome smoothness to new galaxy ai feautersall package this phoneVALU FOR MONEYI DONT HAVE ANY WORDS\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Vilas N Patil\", \"rating\": \"5.0\", \"date\": \"26 May 2025\", \"text\": \"Nice product and received all items as required\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Amazon Customer\", \"rating\": \"5.0\", \"date\": \"23 Apr 2025\", \"text\": \"Awesome phone. Quality make and good looking too.\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Gangadhar\", \"rating\": \"5.0\", \"date\": \"06 May 2025\", \"text\": \"(function() {\n            P.when(\'cr-A\', \'ready\').execute(function(A) {\n                if(typeof A.toggleExpanderAriaLabel === \'function\') {\n                    A.toggleExpanderAriaLabel(\'review_text_read_more\', \'Read more of this review\', \'Read less of this review\');\n                }\n            });\n        })();\n    \n    \n        .review-text-read-more-expander:focus-visible {\n            outline: 2px solid #2162a1;\n            outline-offset: 2px;\n            border-radius: 5px;\n        }\n    \n\n\n\n\n\n\n\n\n  \n  \n    Exceptional photo quality great processerBest in the segment display most optimized software  value got money in this price range.Great fast charging no noticeable heating issues but gets temperature\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Thomas\", \"rating\": \"5.0\", \"date\": \"16 May 2025\", \"text\": \"Bought it for 35kTotally worth it for 35k a phone with flagship features camera is very nice you get 4k recording on all 4 camera for this price it\'s pretty rare but on one UI 6.1 it had some heating issue but after updating to oneui7 it stopped heating so much it has far far better heat mangement than s23fe and also chin is slightly thick but most of the time you won\'t notice it gaming is smooth and I get 60fps most of the time you get extrem plus on bgmi\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Abhishek katoch\", \"rating\": \"4.0\", \"date\": \"18 May 2025\", \"text\": \"Device is really good . The only issue is heating\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Annappa\", \"rating\": \"1.0\", \"date\": \"22 May 2025\", \"text\": \"Please don\'t buy these expensive mobiles from Amazon, After paying hell amount of money, you need to run behind service centres for new phone service.\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"negative\"}, {\"author\": \"Ramiz mariner\", \"rating\": \"5.0\", \"date\": \"04 Mar 2025\", \"text\": \"Writing the review after 10 days of usage.Phone Quality - quality is just awesome, looks premium.Size- this matters person to person, honestly I love to have phone size of 5.5 or even 5.0, but know you don\'t get such small size Phone. Coming back to this, I am 5.10 ft, so for my hand this mobile looks big, unable to use with one hand.Performance- have played games continously, watched champions trophy.. Performance is very good...Battery life - it good enough to survive for all day.Weight- again this comes person to person, I l9ve the weight of this cell phone, quiet heavy....\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"RAAZ PATHAN\", \"rating\": \"5.0\", \"date\": \"20 May 2025\", \"text\": \"awesome smoothness to new galaxy ai feautersall package this phoneVALU FOR MONEYI DONT HAVE ANY WORDS\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Vilas N Patil\", \"rating\": \"5.0\", \"date\": \"26 May 2025\", \"text\": \"Nice product and received all items as required\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}, {\"author\": \"Amazon Customer\", \"rating\": \"5.0\", \"date\": \"23 Apr 2025\", \"text\": \"Awesome phone. Quality make and good looking too.\n  \nRead more\", \"product_id\": \"B0DHL7YT5S\", \"link\": \"https://www.amazon.in/Samsung-Galaxy-Smartphone-Graphite-Storage/dp/B0DHL7YT5S/ref=sr_1_3?crid=2RBF62FWJ6B00&amp;dib=eyJ2IjoiMSJ9.0BWpZ4ImHW1ZfRnJShi1zt8rS2ZXr8WafZOkgOSNJy6ZEfZ1hwYeKXLo-_RuJx_SP6q3kZ5oHy2xRo6ULiehbeSwws5GCN1AbOWSwhpcPah50e9AED9-5JAS7BMHO8KvX4o_dnRI6mUlkSQwtEdNDqZG81K-wfO7o8zA0-Ox-qKK7OA56W4NHuA6-8FyspcAJjF5yeHBAqIAKEPxDIVNR8aemN5h3BAsdzOTg1zQdXo.qL_kbcmjSDyS6paC8Fc_O02S9a0gPjjgIlZtBHkM4Vs&amp;dib_tag=se&amp;keywords=samsung+s24+fe+5g&amp;qid=1748537484&amp;sprefix=samsun,aps,255&amp;sr=8-3\", \"sentiment\": \"positive\"}]}</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">

</xml_diff>